<commit_message>
fix for tmp and the shapes
</commit_message>
<xml_diff>
--- a/Greyform/Python_Application/exporteddatassss(with TMP)(draft)(tetra).xlsx
+++ b/Greyform/Python_Application/exporteddatassss(with TMP)(draft)(tetra).xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="107">
   <si>
     <t>Marking type</t>
   </si>
@@ -63,226 +63,232 @@
     <t>Tile</t>
   </si>
   <si>
-    <t>TMP1S2a4:TMP1S2a4:1155192</t>
-  </si>
-  <si>
-    <t>TMP1S2f1:TMP1S2f1:1155220</t>
-  </si>
-  <si>
-    <t>TMP1S2f2:TMP1S2f2:1155219</t>
-  </si>
-  <si>
-    <t>TMP1S2f3:TMP1S2f3:1155218</t>
-  </si>
-  <si>
-    <t>TMP1S2e1:TMP1S2e1:1155215</t>
-  </si>
-  <si>
-    <t>TMP1S2e2:TMP1S2e2:1155214</t>
-  </si>
-  <si>
-    <t>TMP1S2e3:TMP1S2e3:1155213</t>
-  </si>
-  <si>
-    <t>TMP1S2e4:TMP1S2e4:1155212</t>
-  </si>
-  <si>
-    <t>TMP1S2d1:TMP1S2d1:1155210</t>
-  </si>
-  <si>
-    <t>TMP1S2d2:TMP1S2d2:1155209</t>
-  </si>
-  <si>
-    <t>TMP1S2d3:TMP1S2d3:1155208</t>
-  </si>
-  <si>
-    <t>TMP1S2d4:TMP1S2d4:1155207</t>
-  </si>
-  <si>
-    <t>TMP1S2f4:TMP1S2f4:1155217</t>
-  </si>
-  <si>
-    <t>TMP1S2c2:TMP1S2c2:1155204</t>
-  </si>
-  <si>
-    <t>TMP1S2c3:TMP1S2c3:1155203</t>
-  </si>
-  <si>
-    <t>TMP1S2c4:TMP1S2c4:1155202</t>
-  </si>
-  <si>
-    <t>TMP1S2b1:TMP1S2b1:1155200</t>
-  </si>
-  <si>
-    <t>TMP1S2b2:TMP1S2b2:1155199</t>
-  </si>
-  <si>
-    <t>TMP1S2b3:TMP1S2b3:1155198</t>
-  </si>
-  <si>
-    <t>TMP1S2b4:TMP1S2b4:1155197</t>
-  </si>
-  <si>
-    <t>TMP1S2a1:TMP1S2a1:1155195</t>
-  </si>
-  <si>
-    <t>TMP1S2a2:TMP1S2a2:1155194</t>
-  </si>
-  <si>
-    <t>TMP1S2a3:TMP1S2a3:1155193</t>
-  </si>
-  <si>
-    <t>TMP1S2c1:TMP1S2c1:1155205</t>
-  </si>
-  <si>
-    <t>TMP2S2c2:TMP2S2c2:1156962</t>
-  </si>
-  <si>
-    <t>TMP2S2c1:TMP2S2c1:1156963</t>
-  </si>
-  <si>
-    <t>TMP2S2a1:TMP2S2a1:1155225</t>
-  </si>
-  <si>
-    <t>TMP2S2b1:TMP2S2b1:1155223</t>
-  </si>
-  <si>
-    <t>TMP2S2b2:TMP2S2b2:1155222</t>
-  </si>
-  <si>
-    <t>TMP2S2a2:TMP2S2a2:1155224</t>
-  </si>
-  <si>
-    <t>TMP3S2b4:TMP3S2b4:1155227</t>
-  </si>
-  <si>
-    <t>TMP3S2b3:TMP3S2b3:1155228</t>
-  </si>
-  <si>
-    <t>TMP3S2b1:TMP3S2b1:1155229</t>
-  </si>
-  <si>
-    <t>TMP3S2b2:TMP3S2b2:1155230</t>
-  </si>
-  <si>
-    <t>TMP3S2a4:TMP3S2a4:1155231</t>
-  </si>
-  <si>
-    <t>TMP3S2a3:TMP3S2a3:1155232</t>
-  </si>
-  <si>
-    <t>TMP3S2a2:TMP3S2a2:1155233</t>
-  </si>
-  <si>
-    <t>TMP3S2a1:TMP3S2a1:1155234</t>
-  </si>
-  <si>
-    <t>TMP4S2a1:TMP4S2a1:1155243</t>
-  </si>
-  <si>
-    <t>TMP4S2a2:TMP4S2a2:1155242</t>
-  </si>
-  <si>
-    <t>TMP4S2b1:TMP4S2b1:1155240</t>
-  </si>
-  <si>
-    <t>TMP4S2b2:TMP4S2b2:1155239</t>
-  </si>
-  <si>
-    <t>TMP4S2b4:TMP4S2b4:1155236</t>
-  </si>
-  <si>
-    <t>TMP4S2a4:TMP4S2a4:1155237</t>
-  </si>
-  <si>
-    <t>TMP4S2b3:TMP4S2b3:1155238</t>
-  </si>
-  <si>
-    <t>TMP4S2a3:TMP4S2a3:1155241</t>
-  </si>
-  <si>
-    <t>TMP5S2a1:TMP5S2a1:1155252</t>
-  </si>
-  <si>
-    <t>TMP5S2b1:TMP5S2b1:1155251</t>
-  </si>
-  <si>
-    <t>TMP5S2a2:TMP5S2a2:1155249</t>
-  </si>
-  <si>
-    <t>TMP5S2a3:TMP5S2a3:1155247</t>
-  </si>
-  <si>
-    <t>TMP5S2b4:TMP5S2b4:1155246</t>
-  </si>
-  <si>
-    <t>TMP5S2b3:TMP5S2b3:1155248</t>
-  </si>
-  <si>
-    <t>TMP5S2b2:TMP5S2b2:1155250</t>
-  </si>
-  <si>
-    <t>TMP5S2a4:TMP5S2a4:1155245</t>
-  </si>
-  <si>
-    <t>TMP6S2a3:TMP6S2a3:1155254</t>
-  </si>
-  <si>
-    <t>TMP6S2a4:TMP6S2a4:1155255</t>
-  </si>
-  <si>
-    <t>TMP6S2a2:TMP6S2a2:1155256</t>
-  </si>
-  <si>
-    <t>TMP6S2a1:TMP6S2a1:1155257</t>
-  </si>
-  <si>
-    <t>TMP6S2b4:TMP6S2b4:1155259</t>
-  </si>
-  <si>
-    <t>TMP6S2b3:TMP6S2b3:1155260</t>
-  </si>
-  <si>
-    <t>TMP6S2b2:TMP6S2b2:1155261</t>
-  </si>
-  <si>
-    <t>TMP6S2b1:TMP6S2b1:1155262</t>
-  </si>
-  <si>
-    <t>TMP7S2c1:TMP7S2c1:1155276</t>
-  </si>
-  <si>
-    <t>TMP7S2d1:TMP7S2d1:1155271</t>
-  </si>
-  <si>
-    <t>TMP7S2c3:TMP7S2c3:1155274</t>
-  </si>
-  <si>
-    <t>TMP7S2d3:TMP7S2d3:1155273</t>
-  </si>
-  <si>
-    <t>TMP7S2d2:TMP7S2d2:1155272</t>
-  </si>
-  <si>
-    <t>TMP7S2a1:TMP7S2a1:1155269</t>
-  </si>
-  <si>
-    <t>TMP7S2a2:TMP7S2a2:1155268</t>
-  </si>
-  <si>
-    <t>TMP7S2a3:TMP7S2a3:1155267</t>
-  </si>
-  <si>
-    <t>TMP7S2b2:TMP7S2b2:1155265</t>
-  </si>
-  <si>
-    <t>TMP7S2b3:TMP7S2b3:1155264</t>
-  </si>
-  <si>
-    <t>TMP7S2c2:TMP7S2c2:1155275</t>
-  </si>
-  <si>
-    <t>TMP7S2b1:TMP7S2b1:1155266</t>
+    <t>TMP1S2c2</t>
+  </si>
+  <si>
+    <t>TMP1S2d3</t>
+  </si>
+  <si>
+    <t>TMP1S2d2</t>
+  </si>
+  <si>
+    <t>TMP1S2d1</t>
+  </si>
+  <si>
+    <t>TMP1S2c4</t>
+  </si>
+  <si>
+    <t>TMP1S2c3</t>
+  </si>
+  <si>
+    <t>TMP1S2e2</t>
+  </si>
+  <si>
+    <t>TMP1S2c1</t>
+  </si>
+  <si>
+    <t>TMP1S2b4</t>
+  </si>
+  <si>
+    <t>TMP1S2b3</t>
+  </si>
+  <si>
+    <t>TMP1S2b2</t>
+  </si>
+  <si>
+    <t>TMP1S2d4</t>
+  </si>
+  <si>
+    <t>TMP1S2b1</t>
+  </si>
+  <si>
+    <t>TMP1S2a3</t>
+  </si>
+  <si>
+    <t>TMP1S2a2</t>
+  </si>
+  <si>
+    <t>TMP1S2a1</t>
+  </si>
+  <si>
+    <t>TMP1S2e3</t>
+  </si>
+  <si>
+    <t>TMP1S2e4</t>
+  </si>
+  <si>
+    <t>TMP1S2f1</t>
+  </si>
+  <si>
+    <t>TMP1S2f2</t>
+  </si>
+  <si>
+    <t>TMP1S2f3</t>
+  </si>
+  <si>
+    <t>TMP1S2f4</t>
+  </si>
+  <si>
+    <t>TMP1S2a4</t>
+  </si>
+  <si>
+    <t>TMP1S2e1</t>
+  </si>
+  <si>
+    <t>TMP2S2c1</t>
+  </si>
+  <si>
+    <t>TMP2S2c3</t>
+  </si>
+  <si>
+    <t>TMP2S2c2</t>
+  </si>
+  <si>
+    <t>TMP2S2c4</t>
+  </si>
+  <si>
+    <t>TMP3S2a1</t>
+  </si>
+  <si>
+    <t>TMP3S2a2</t>
+  </si>
+  <si>
+    <t>TMP3S2a3</t>
+  </si>
+  <si>
+    <t>TMP3S2a4</t>
+  </si>
+  <si>
+    <t>TMP3S2b1</t>
+  </si>
+  <si>
+    <t>TMP3S2b3</t>
+  </si>
+  <si>
+    <t>TMP3S2b4</t>
+  </si>
+  <si>
+    <t>TMP3S2b2</t>
+  </si>
+  <si>
+    <t>TMP4S2b4</t>
+  </si>
+  <si>
+    <t>TMP4S2b3</t>
+  </si>
+  <si>
+    <t>TMP4S2a1</t>
+  </si>
+  <si>
+    <t>TMP4S2a2</t>
+  </si>
+  <si>
+    <t>TMP4S2a3</t>
+  </si>
+  <si>
+    <t>TMP4S2a4</t>
+  </si>
+  <si>
+    <t>TMP4S2b1</t>
+  </si>
+  <si>
+    <t>TMP4S2b2</t>
+  </si>
+  <si>
+    <t>TMP5S2a4</t>
+  </si>
+  <si>
+    <t>TMP5S2a3</t>
+  </si>
+  <si>
+    <t>TMP5S2a2</t>
+  </si>
+  <si>
+    <t>TMP5S2a1</t>
+  </si>
+  <si>
+    <t>TMP6S2b1</t>
+  </si>
+  <si>
+    <t>TMP6S2a1</t>
+  </si>
+  <si>
+    <t>TMP6S2a2</t>
+  </si>
+  <si>
+    <t>TMP6S2a3</t>
+  </si>
+  <si>
+    <t>TMP6S2a4</t>
+  </si>
+  <si>
+    <t>TMP6S2b4</t>
+  </si>
+  <si>
+    <t>TMP6S2b2</t>
+  </si>
+  <si>
+    <t>TMP6S2b3</t>
+  </si>
+  <si>
+    <t>TMP7S2b3</t>
+  </si>
+  <si>
+    <t>TMP7S2b4</t>
+  </si>
+  <si>
+    <t>TMP7S2b5</t>
+  </si>
+  <si>
+    <t>TMP7S2b6</t>
+  </si>
+  <si>
+    <t>TMP7S2b7</t>
+  </si>
+  <si>
+    <t>TMP7S2c1</t>
+  </si>
+  <si>
+    <t>TMP7S2c2</t>
+  </si>
+  <si>
+    <t>TMP7S2d1</t>
+  </si>
+  <si>
+    <t>TMP7S2b2</t>
+  </si>
+  <si>
+    <t>TMP7S2d2</t>
+  </si>
+  <si>
+    <t>TMP7S2b1</t>
+  </si>
+  <si>
+    <t>TMP7S2a6</t>
+  </si>
+  <si>
+    <t>TMP7S2a5</t>
+  </si>
+  <si>
+    <t>TMP7S2a4</t>
+  </si>
+  <si>
+    <t>TMP7S2a3</t>
+  </si>
+  <si>
+    <t>TMP7S2a2</t>
+  </si>
+  <si>
+    <t>TMP7S2a1</t>
+  </si>
+  <si>
+    <t>TMP7S2e1</t>
+  </si>
+  <si>
+    <t>TMP7S2a7</t>
+  </si>
+  <si>
+    <t>TMP7S2e2</t>
   </si>
   <si>
     <t>F</t>
@@ -297,12 +303,12 @@
     <t>Fitting</t>
   </si>
   <si>
+    <t>BSS.HAND SHOWER SET.MASTER BATH:BSS.HAND SHOWER SET.MASTER BATH:1091130</t>
+  </si>
+  <si>
     <t>BSS.GESSI.SM.49079:29046000:1090989</t>
   </si>
   <si>
-    <t>BSS.HAND SHOWER SET.MASTER BATH:BSS.HAND SHOWER SET.MASTER BATH:1091130</t>
-  </si>
-  <si>
     <t>BSS.MIRROR CABINET.C5-MASTER BATH:BSS.MIRROR CABINET.C5-MASTER BATH:1090945</t>
   </si>
   <si>
@@ -312,10 +318,10 @@
     <t>BSS.LAUFEN.WC.820714:820959000 White:1091064</t>
   </si>
   <si>
+    <t>BSS.TECE.AP.9240402:Flush Plate:1091024</t>
+  </si>
+  <si>
     <t>BSS.GESSI,BM.49001:Default:1090988</t>
-  </si>
-  <si>
-    <t>BSS.TECE.AP.9240402:Flush Plate:1091024</t>
   </si>
   <si>
     <t>BSS.MONIC.BIB TAP.T-4L:BIB TAP:1090961</t>
@@ -688,7 +694,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O75"/>
+  <dimension ref="A1:O77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:15">
@@ -737,7 +743,7 @@
     </row>
     <row r="2" spans="1:15">
       <c r="A2" s="1">
-        <v>10</v>
+        <v>174</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
@@ -749,10 +755,10 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>-1.35</v>
+        <v>0.47</v>
       </c>
       <c r="F2">
-        <v>-0.775</v>
+        <v>-0.175</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -761,7 +767,7 @@
         <v>1</v>
       </c>
       <c r="I2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -775,7 +781,7 @@
     </row>
     <row r="3" spans="1:15">
       <c r="A3" s="1">
-        <v>33</v>
+        <v>179</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -787,10 +793,10 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>0.9350000000000001</v>
+        <v>-0.03</v>
       </c>
       <c r="F3">
-        <v>1.025</v>
+        <v>0.425</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -799,7 +805,7 @@
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -813,7 +819,7 @@
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="1">
-        <v>32</v>
+        <v>178</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
@@ -825,10 +831,10 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>0.9350000000000001</v>
+        <v>-0.03</v>
       </c>
       <c r="F4">
-        <v>0.425</v>
+        <v>-0.175</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -837,7 +843,7 @@
         <v>1</v>
       </c>
       <c r="I4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -851,7 +857,7 @@
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="1">
-        <v>31</v>
+        <v>177</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
@@ -863,10 +869,10 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>0.9350000000000001</v>
+        <v>-0.03</v>
       </c>
       <c r="F5">
-        <v>-0.175</v>
+        <v>-0.775</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -875,7 +881,7 @@
         <v>1</v>
       </c>
       <c r="I5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -889,7 +895,7 @@
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="1">
-        <v>29</v>
+        <v>176</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
@@ -901,7 +907,7 @@
         <v>0</v>
       </c>
       <c r="E6">
-        <v>0.49</v>
+        <v>0.47</v>
       </c>
       <c r="F6">
         <v>1.025</v>
@@ -913,7 +919,7 @@
         <v>1</v>
       </c>
       <c r="I6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -927,7 +933,7 @@
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="1">
-        <v>28</v>
+        <v>175</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -939,7 +945,7 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <v>0.49</v>
+        <v>0.47</v>
       </c>
       <c r="F7">
         <v>0.425</v>
@@ -951,7 +957,7 @@
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -965,7 +971,7 @@
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="1">
-        <v>27</v>
+        <v>182</v>
       </c>
       <c r="B8" t="s">
         <v>14</v>
@@ -977,7 +983,7 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>0.49</v>
+        <v>-0.35</v>
       </c>
       <c r="F8">
         <v>-0.175</v>
@@ -989,7 +995,7 @@
         <v>1</v>
       </c>
       <c r="I8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -1003,7 +1009,7 @@
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="1">
-        <v>26</v>
+        <v>173</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
@@ -1015,10 +1021,10 @@
         <v>0</v>
       </c>
       <c r="E9">
-        <v>0.49</v>
+        <v>0.47</v>
       </c>
       <c r="F9">
-        <v>1.025</v>
+        <v>-0.775</v>
       </c>
       <c r="G9">
         <v>1</v>
@@ -1027,7 +1033,7 @@
         <v>1</v>
       </c>
       <c r="I9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J9">
         <v>1</v>
@@ -1041,7 +1047,7 @@
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="1">
-        <v>25</v>
+        <v>172</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
@@ -1053,7 +1059,7 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>0.47</v>
+        <v>0.49</v>
       </c>
       <c r="F10">
         <v>1.025</v>
@@ -1065,7 +1071,7 @@
         <v>1</v>
       </c>
       <c r="I10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J10">
         <v>1</v>
@@ -1079,7 +1085,7 @@
     </row>
     <row r="11" spans="1:15">
       <c r="A11" s="1">
-        <v>24</v>
+        <v>171</v>
       </c>
       <c r="B11" t="s">
         <v>14</v>
@@ -1091,7 +1097,7 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>0.47</v>
+        <v>0.49</v>
       </c>
       <c r="F11">
         <v>0.425</v>
@@ -1103,7 +1109,7 @@
         <v>1</v>
       </c>
       <c r="I11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J11">
         <v>1</v>
@@ -1117,7 +1123,7 @@
     </row>
     <row r="12" spans="1:15">
       <c r="A12" s="1">
-        <v>23</v>
+        <v>170</v>
       </c>
       <c r="B12" t="s">
         <v>14</v>
@@ -1129,7 +1135,7 @@
         <v>0</v>
       </c>
       <c r="E12">
-        <v>0.47</v>
+        <v>0.49</v>
       </c>
       <c r="F12">
         <v>-0.175</v>
@@ -1141,7 +1147,7 @@
         <v>1</v>
       </c>
       <c r="I12" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J12">
         <v>1</v>
@@ -1155,7 +1161,7 @@
     </row>
     <row r="13" spans="1:15">
       <c r="A13" s="1">
-        <v>22</v>
+        <v>180</v>
       </c>
       <c r="B13" t="s">
         <v>14</v>
@@ -1167,10 +1173,10 @@
         <v>0</v>
       </c>
       <c r="E13">
-        <v>0.47</v>
+        <v>-0.03</v>
       </c>
       <c r="F13">
-        <v>-0.775</v>
+        <v>1.025</v>
       </c>
       <c r="G13">
         <v>1</v>
@@ -1179,7 +1185,7 @@
         <v>1</v>
       </c>
       <c r="I13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J13">
         <v>1</v>
@@ -1193,7 +1199,7 @@
     </row>
     <row r="14" spans="1:15">
       <c r="A14" s="1">
-        <v>30</v>
+        <v>169</v>
       </c>
       <c r="B14" t="s">
         <v>14</v>
@@ -1205,7 +1211,7 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>0.9350000000000001</v>
+        <v>0.49</v>
       </c>
       <c r="F14">
         <v>-0.775</v>
@@ -1217,7 +1223,7 @@
         <v>1</v>
       </c>
       <c r="I14" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J14">
         <v>1</v>
@@ -1231,7 +1237,7 @@
     </row>
     <row r="15" spans="1:15">
       <c r="A15" s="1">
-        <v>20</v>
+        <v>167</v>
       </c>
       <c r="B15" t="s">
         <v>14</v>
@@ -1243,7 +1249,7 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>-0.03</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F15">
         <v>0.425</v>
@@ -1255,7 +1261,7 @@
         <v>1</v>
       </c>
       <c r="I15" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J15">
         <v>1</v>
@@ -1269,7 +1275,7 @@
     </row>
     <row r="16" spans="1:15">
       <c r="A16" s="1">
-        <v>19</v>
+        <v>166</v>
       </c>
       <c r="B16" t="s">
         <v>14</v>
@@ -1281,7 +1287,7 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>-0.03</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F16">
         <v>-0.175</v>
@@ -1293,7 +1299,7 @@
         <v>1</v>
       </c>
       <c r="I16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J16">
         <v>1</v>
@@ -1307,7 +1313,7 @@
     </row>
     <row r="17" spans="1:13">
       <c r="A17" s="1">
-        <v>18</v>
+        <v>165</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
@@ -1319,7 +1325,7 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>-0.03</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F17">
         <v>-0.775</v>
@@ -1331,7 +1337,7 @@
         <v>1</v>
       </c>
       <c r="I17" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J17">
         <v>1</v>
@@ -1345,7 +1351,7 @@
     </row>
     <row r="18" spans="1:13">
       <c r="A18" s="1">
-        <v>17</v>
+        <v>183</v>
       </c>
       <c r="B18" t="s">
         <v>14</v>
@@ -1360,7 +1366,7 @@
         <v>-0.35</v>
       </c>
       <c r="F18">
-        <v>1.025</v>
+        <v>0.425</v>
       </c>
       <c r="G18">
         <v>1</v>
@@ -1369,7 +1375,7 @@
         <v>1</v>
       </c>
       <c r="I18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J18">
         <v>1</v>
@@ -1383,7 +1389,7 @@
     </row>
     <row r="19" spans="1:13">
       <c r="A19" s="1">
-        <v>16</v>
+        <v>184</v>
       </c>
       <c r="B19" t="s">
         <v>14</v>
@@ -1398,7 +1404,7 @@
         <v>-0.35</v>
       </c>
       <c r="F19">
-        <v>0.425</v>
+        <v>1.025</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -1407,7 +1413,7 @@
         <v>1</v>
       </c>
       <c r="I19" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J19">
         <v>1</v>
@@ -1421,7 +1427,7 @@
     </row>
     <row r="20" spans="1:13">
       <c r="A20" s="1">
-        <v>15</v>
+        <v>185</v>
       </c>
       <c r="B20" t="s">
         <v>14</v>
@@ -1433,10 +1439,10 @@
         <v>0</v>
       </c>
       <c r="E20">
-        <v>-0.35</v>
+        <v>-1.35</v>
       </c>
       <c r="F20">
-        <v>-0.175</v>
+        <v>-0.775</v>
       </c>
       <c r="G20">
         <v>1</v>
@@ -1445,7 +1451,7 @@
         <v>1</v>
       </c>
       <c r="I20" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J20">
         <v>1</v>
@@ -1459,7 +1465,7 @@
     </row>
     <row r="21" spans="1:13">
       <c r="A21" s="1">
-        <v>14</v>
+        <v>186</v>
       </c>
       <c r="B21" t="s">
         <v>14</v>
@@ -1471,10 +1477,10 @@
         <v>0</v>
       </c>
       <c r="E21">
-        <v>-0.35</v>
+        <v>-1.35</v>
       </c>
       <c r="F21">
-        <v>-0.775</v>
+        <v>-0.175</v>
       </c>
       <c r="G21">
         <v>1</v>
@@ -1483,7 +1489,7 @@
         <v>1</v>
       </c>
       <c r="I21" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J21">
         <v>1</v>
@@ -1497,7 +1503,7 @@
     </row>
     <row r="22" spans="1:13">
       <c r="A22" s="1">
-        <v>13</v>
+        <v>187</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
@@ -1512,7 +1518,7 @@
         <v>-1.35</v>
       </c>
       <c r="F22">
-        <v>1.025</v>
+        <v>0.425</v>
       </c>
       <c r="G22">
         <v>1</v>
@@ -1521,7 +1527,7 @@
         <v>1</v>
       </c>
       <c r="I22" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J22">
         <v>1</v>
@@ -1535,7 +1541,7 @@
     </row>
     <row r="23" spans="1:13">
       <c r="A23" s="1">
-        <v>12</v>
+        <v>188</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
@@ -1550,7 +1556,7 @@
         <v>-1.35</v>
       </c>
       <c r="F23">
-        <v>0.425</v>
+        <v>1.025</v>
       </c>
       <c r="G23">
         <v>1</v>
@@ -1559,7 +1565,7 @@
         <v>1</v>
       </c>
       <c r="I23" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J23">
         <v>1</v>
@@ -1573,7 +1579,7 @@
     </row>
     <row r="24" spans="1:13">
       <c r="A24" s="1">
-        <v>11</v>
+        <v>168</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
@@ -1585,10 +1591,10 @@
         <v>0</v>
       </c>
       <c r="E24">
-        <v>-1.35</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F24">
-        <v>-0.175</v>
+        <v>1.025</v>
       </c>
       <c r="G24">
         <v>1</v>
@@ -1597,7 +1603,7 @@
         <v>1</v>
       </c>
       <c r="I24" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J24">
         <v>1</v>
@@ -1611,7 +1617,7 @@
     </row>
     <row r="25" spans="1:13">
       <c r="A25" s="1">
-        <v>21</v>
+        <v>181</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
@@ -1623,10 +1629,10 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>-0.03</v>
+        <v>-0.35</v>
       </c>
       <c r="F25">
-        <v>1.025</v>
+        <v>-0.775</v>
       </c>
       <c r="G25">
         <v>1</v>
@@ -1635,7 +1641,7 @@
         <v>1</v>
       </c>
       <c r="I25" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J25">
         <v>1</v>
@@ -1649,7 +1655,7 @@
     </row>
     <row r="26" spans="1:13">
       <c r="A26" s="1">
-        <v>82</v>
+        <v>189</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
@@ -1658,13 +1664,13 @@
         <v>39</v>
       </c>
       <c r="D26">
-        <v>2.76</v>
+        <v>0</v>
       </c>
       <c r="E26">
         <v>0.15</v>
       </c>
       <c r="F26">
-        <v>0.425</v>
+        <v>-0.775</v>
       </c>
       <c r="G26">
         <v>2</v>
@@ -1673,7 +1679,7 @@
         <v>1</v>
       </c>
       <c r="I26" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J26">
         <v>1</v>
@@ -1687,7 +1693,7 @@
     </row>
     <row r="27" spans="1:13">
       <c r="A27" s="1">
-        <v>83</v>
+        <v>191</v>
       </c>
       <c r="B27" t="s">
         <v>14</v>
@@ -1696,13 +1702,13 @@
         <v>40</v>
       </c>
       <c r="D27">
-        <v>2.76</v>
+        <v>0</v>
       </c>
       <c r="E27">
         <v>0.15</v>
       </c>
       <c r="F27">
-        <v>1.025</v>
+        <v>0.425</v>
       </c>
       <c r="G27">
         <v>2</v>
@@ -1711,7 +1717,7 @@
         <v>1</v>
       </c>
       <c r="I27" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J27">
         <v>1</v>
@@ -1725,7 +1731,7 @@
     </row>
     <row r="28" spans="1:13">
       <c r="A28" s="1">
-        <v>37</v>
+        <v>190</v>
       </c>
       <c r="B28" t="s">
         <v>14</v>
@@ -1734,10 +1740,10 @@
         <v>41</v>
       </c>
       <c r="D28">
-        <v>2.76</v>
+        <v>0</v>
       </c>
       <c r="E28">
-        <v>-0.5</v>
+        <v>0.15</v>
       </c>
       <c r="F28">
         <v>-0.175</v>
@@ -1749,7 +1755,7 @@
         <v>1</v>
       </c>
       <c r="I28" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J28">
         <v>1</v>
@@ -1763,7 +1769,7 @@
     </row>
     <row r="29" spans="1:13">
       <c r="A29" s="1">
-        <v>35</v>
+        <v>192</v>
       </c>
       <c r="B29" t="s">
         <v>14</v>
@@ -1772,13 +1778,13 @@
         <v>42</v>
       </c>
       <c r="D29">
-        <v>2.76</v>
+        <v>0</v>
       </c>
       <c r="E29">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F29">
-        <v>-0.175</v>
+        <v>1.025</v>
       </c>
       <c r="G29">
         <v>2</v>
@@ -1787,7 +1793,7 @@
         <v>1</v>
       </c>
       <c r="I29" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J29">
         <v>1</v>
@@ -1801,7 +1807,7 @@
     </row>
     <row r="30" spans="1:13">
       <c r="A30" s="1">
-        <v>34</v>
+        <v>193</v>
       </c>
       <c r="B30" t="s">
         <v>14</v>
@@ -1810,28 +1816,28 @@
         <v>43</v>
       </c>
       <c r="D30">
-        <v>2.76</v>
+        <v>0.6</v>
       </c>
       <c r="E30">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="F30">
         <v>-0.775</v>
       </c>
       <c r="G30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H30">
         <v>1</v>
       </c>
       <c r="I30" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J30">
         <v>1</v>
       </c>
       <c r="L30">
-        <v>1.34</v>
+        <v>0.96</v>
       </c>
       <c r="M30">
         <v>2.655</v>
@@ -1839,7 +1845,7 @@
     </row>
     <row r="31" spans="1:13">
       <c r="A31" s="1">
-        <v>36</v>
+        <v>194</v>
       </c>
       <c r="B31" t="s">
         <v>14</v>
@@ -1848,28 +1854,28 @@
         <v>44</v>
       </c>
       <c r="D31">
-        <v>2.76</v>
+        <v>0.6</v>
       </c>
       <c r="E31">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="F31">
-        <v>-0.775</v>
+        <v>-0.175</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H31">
         <v>1</v>
       </c>
       <c r="I31" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J31">
         <v>1</v>
       </c>
       <c r="L31">
-        <v>1.34</v>
+        <v>0.96</v>
       </c>
       <c r="M31">
         <v>2.655</v>
@@ -1877,7 +1883,7 @@
     </row>
     <row r="32" spans="1:13">
       <c r="A32" s="1">
-        <v>38</v>
+        <v>195</v>
       </c>
       <c r="B32" t="s">
         <v>14</v>
@@ -1886,13 +1892,13 @@
         <v>45</v>
       </c>
       <c r="D32">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="E32">
-        <v>0.445</v>
+        <v>0</v>
       </c>
       <c r="F32">
-        <v>-0.775</v>
+        <v>0.425</v>
       </c>
       <c r="G32">
         <v>3</v>
@@ -1901,7 +1907,7 @@
         <v>1</v>
       </c>
       <c r="I32" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J32">
         <v>1</v>
@@ -1915,7 +1921,7 @@
     </row>
     <row r="33" spans="1:13">
       <c r="A33" s="1">
-        <v>39</v>
+        <v>196</v>
       </c>
       <c r="B33" t="s">
         <v>14</v>
@@ -1924,13 +1930,13 @@
         <v>46</v>
       </c>
       <c r="D33">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="E33">
-        <v>0.445</v>
+        <v>0</v>
       </c>
       <c r="F33">
-        <v>-0.175</v>
+        <v>1.025</v>
       </c>
       <c r="G33">
         <v>3</v>
@@ -1939,7 +1945,7 @@
         <v>1</v>
       </c>
       <c r="I33" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J33">
         <v>1</v>
@@ -1953,7 +1959,7 @@
     </row>
     <row r="34" spans="1:13">
       <c r="A34" s="1">
-        <v>40</v>
+        <v>197</v>
       </c>
       <c r="B34" t="s">
         <v>14</v>
@@ -1962,13 +1968,13 @@
         <v>47</v>
       </c>
       <c r="D34">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="E34">
         <v>0.445</v>
       </c>
       <c r="F34">
-        <v>1.025</v>
+        <v>-0.775</v>
       </c>
       <c r="G34">
         <v>3</v>
@@ -1977,7 +1983,7 @@
         <v>1</v>
       </c>
       <c r="I34" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J34">
         <v>1</v>
@@ -1991,7 +1997,7 @@
     </row>
     <row r="35" spans="1:13">
       <c r="A35" s="1">
-        <v>41</v>
+        <v>199</v>
       </c>
       <c r="B35" t="s">
         <v>14</v>
@@ -2000,7 +2006,7 @@
         <v>48</v>
       </c>
       <c r="D35">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="E35">
         <v>0.445</v>
@@ -2015,7 +2021,7 @@
         <v>1</v>
       </c>
       <c r="I35" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J35">
         <v>1</v>
@@ -2029,7 +2035,7 @@
     </row>
     <row r="36" spans="1:13">
       <c r="A36" s="1">
-        <v>42</v>
+        <v>200</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
@@ -2038,10 +2044,10 @@
         <v>49</v>
       </c>
       <c r="D36">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>0.445</v>
       </c>
       <c r="F36">
         <v>1.025</v>
@@ -2053,7 +2059,7 @@
         <v>1</v>
       </c>
       <c r="I36" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J36">
         <v>1</v>
@@ -2067,7 +2073,7 @@
     </row>
     <row r="37" spans="1:13">
       <c r="A37" s="1">
-        <v>43</v>
+        <v>198</v>
       </c>
       <c r="B37" t="s">
         <v>14</v>
@@ -2076,10 +2082,10 @@
         <v>50</v>
       </c>
       <c r="D37">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="E37">
-        <v>0</v>
+        <v>0.445</v>
       </c>
       <c r="F37">
         <v>-0.175</v>
@@ -2091,7 +2097,7 @@
         <v>1</v>
       </c>
       <c r="I37" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J37">
         <v>1</v>
@@ -2105,7 +2111,7 @@
     </row>
     <row r="38" spans="1:13">
       <c r="A38" s="1">
-        <v>44</v>
+        <v>208</v>
       </c>
       <c r="B38" t="s">
         <v>14</v>
@@ -2114,28 +2120,28 @@
         <v>51</v>
       </c>
       <c r="D38">
-        <v>1.2</v>
+        <v>0.96</v>
       </c>
       <c r="E38">
         <v>0</v>
       </c>
       <c r="F38">
-        <v>0.425</v>
+        <v>1.025</v>
       </c>
       <c r="G38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H38">
         <v>1</v>
       </c>
       <c r="I38" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J38">
         <v>1</v>
       </c>
       <c r="L38">
-        <v>0.96</v>
+        <v>0.592</v>
       </c>
       <c r="M38">
         <v>2.655</v>
@@ -2143,7 +2149,7 @@
     </row>
     <row r="39" spans="1:13">
       <c r="A39" s="1">
-        <v>45</v>
+        <v>207</v>
       </c>
       <c r="B39" t="s">
         <v>14</v>
@@ -2152,28 +2158,28 @@
         <v>52</v>
       </c>
       <c r="D39">
-        <v>1.2</v>
+        <v>0.96</v>
       </c>
       <c r="E39">
         <v>0</v>
       </c>
       <c r="F39">
-        <v>1.025</v>
+        <v>0.425</v>
       </c>
       <c r="G39">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H39">
         <v>1</v>
       </c>
       <c r="I39" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J39">
         <v>1</v>
       </c>
       <c r="L39">
-        <v>0.96</v>
+        <v>0.592</v>
       </c>
       <c r="M39">
         <v>2.655</v>
@@ -2181,7 +2187,7 @@
     </row>
     <row r="40" spans="1:13">
       <c r="A40" s="1">
-        <v>53</v>
+        <v>201</v>
       </c>
       <c r="B40" t="s">
         <v>14</v>
@@ -2190,13 +2196,13 @@
         <v>53</v>
       </c>
       <c r="D40">
-        <v>1.8</v>
+        <v>0.96</v>
       </c>
       <c r="E40">
         <v>-0.3</v>
       </c>
       <c r="F40">
-        <v>1.025</v>
+        <v>-0.775</v>
       </c>
       <c r="G40">
         <v>4</v>
@@ -2205,7 +2211,7 @@
         <v>1</v>
       </c>
       <c r="I40" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J40">
         <v>1</v>
@@ -2219,7 +2225,7 @@
     </row>
     <row r="41" spans="1:13">
       <c r="A41" s="1">
-        <v>52</v>
+        <v>202</v>
       </c>
       <c r="B41" t="s">
         <v>14</v>
@@ -2228,13 +2234,13 @@
         <v>54</v>
       </c>
       <c r="D41">
-        <v>1.8</v>
+        <v>0.96</v>
       </c>
       <c r="E41">
         <v>-0.3</v>
       </c>
       <c r="F41">
-        <v>0.425</v>
+        <v>-0.175</v>
       </c>
       <c r="G41">
         <v>4</v>
@@ -2243,7 +2249,7 @@
         <v>1</v>
       </c>
       <c r="I41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J41">
         <v>1</v>
@@ -2257,7 +2263,7 @@
     </row>
     <row r="42" spans="1:13">
       <c r="A42" s="1">
-        <v>50</v>
+        <v>203</v>
       </c>
       <c r="B42" t="s">
         <v>14</v>
@@ -2266,13 +2272,13 @@
         <v>55</v>
       </c>
       <c r="D42">
-        <v>1.8</v>
+        <v>0.96</v>
       </c>
       <c r="E42">
-        <v>0</v>
+        <v>-0.3</v>
       </c>
       <c r="F42">
-        <v>1.025</v>
+        <v>0.425</v>
       </c>
       <c r="G42">
         <v>4</v>
@@ -2281,7 +2287,7 @@
         <v>1</v>
       </c>
       <c r="I42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J42">
         <v>1</v>
@@ -2295,7 +2301,7 @@
     </row>
     <row r="43" spans="1:13">
       <c r="A43" s="1">
-        <v>49</v>
+        <v>204</v>
       </c>
       <c r="B43" t="s">
         <v>14</v>
@@ -2304,13 +2310,13 @@
         <v>56</v>
       </c>
       <c r="D43">
-        <v>1.8</v>
+        <v>0.96</v>
       </c>
       <c r="E43">
-        <v>0</v>
+        <v>-0.3</v>
       </c>
       <c r="F43">
-        <v>0.425</v>
+        <v>1.025</v>
       </c>
       <c r="G43">
         <v>4</v>
@@ -2319,7 +2325,7 @@
         <v>1</v>
       </c>
       <c r="I43" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J43">
         <v>1</v>
@@ -2333,7 +2339,7 @@
     </row>
     <row r="44" spans="1:13">
       <c r="A44" s="1">
-        <v>46</v>
+        <v>205</v>
       </c>
       <c r="B44" t="s">
         <v>14</v>
@@ -2342,7 +2348,7 @@
         <v>57</v>
       </c>
       <c r="D44">
-        <v>1.8</v>
+        <v>0.96</v>
       </c>
       <c r="E44">
         <v>0</v>
@@ -2357,7 +2363,7 @@
         <v>1</v>
       </c>
       <c r="I44" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J44">
         <v>1</v>
@@ -2371,7 +2377,7 @@
     </row>
     <row r="45" spans="1:13">
       <c r="A45" s="1">
-        <v>47</v>
+        <v>206</v>
       </c>
       <c r="B45" t="s">
         <v>14</v>
@@ -2380,13 +2386,13 @@
         <v>58</v>
       </c>
       <c r="D45">
-        <v>1.8</v>
+        <v>0.96</v>
       </c>
       <c r="E45">
-        <v>-0.3</v>
+        <v>0</v>
       </c>
       <c r="F45">
-        <v>-0.775</v>
+        <v>-0.175</v>
       </c>
       <c r="G45">
         <v>4</v>
@@ -2395,7 +2401,7 @@
         <v>1</v>
       </c>
       <c r="I45" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J45">
         <v>1</v>
@@ -2409,7 +2415,7 @@
     </row>
     <row r="46" spans="1:13">
       <c r="A46" s="1">
-        <v>48</v>
+        <v>212</v>
       </c>
       <c r="B46" t="s">
         <v>14</v>
@@ -2418,28 +2424,28 @@
         <v>59</v>
       </c>
       <c r="D46">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="E46">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="F46">
-        <v>-0.175</v>
+        <v>-0.775</v>
       </c>
       <c r="G46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H46">
         <v>1</v>
       </c>
       <c r="I46" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J46">
         <v>1</v>
       </c>
       <c r="L46">
-        <v>0.592</v>
+        <v>1.94</v>
       </c>
       <c r="M46">
         <v>2.655</v>
@@ -2447,7 +2453,7 @@
     </row>
     <row r="47" spans="1:13">
       <c r="A47" s="1">
-        <v>51</v>
+        <v>211</v>
       </c>
       <c r="B47" t="s">
         <v>14</v>
@@ -2456,28 +2462,28 @@
         <v>60</v>
       </c>
       <c r="D47">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="E47">
-        <v>-0.3</v>
+        <v>0.45</v>
       </c>
       <c r="F47">
-        <v>-0.175</v>
+        <v>-0.775</v>
       </c>
       <c r="G47">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H47">
         <v>1</v>
       </c>
       <c r="I47" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J47">
         <v>1</v>
       </c>
       <c r="L47">
-        <v>0.592</v>
+        <v>1.94</v>
       </c>
       <c r="M47">
         <v>2.655</v>
@@ -2485,7 +2491,7 @@
     </row>
     <row r="48" spans="1:13">
       <c r="A48" s="1">
-        <v>61</v>
+        <v>210</v>
       </c>
       <c r="B48" t="s">
         <v>14</v>
@@ -2494,10 +2500,10 @@
         <v>61</v>
       </c>
       <c r="D48">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="E48">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="F48">
         <v>-0.775</v>
@@ -2509,7 +2515,7 @@
         <v>1</v>
       </c>
       <c r="I48" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J48">
         <v>1</v>
@@ -2523,7 +2529,7 @@
     </row>
     <row r="49" spans="1:13">
       <c r="A49" s="1">
-        <v>60</v>
+        <v>209</v>
       </c>
       <c r="B49" t="s">
         <v>14</v>
@@ -2532,13 +2538,13 @@
         <v>62</v>
       </c>
       <c r="D49">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="E49">
-        <v>0.75</v>
+        <v>-0.45</v>
       </c>
       <c r="F49">
-        <v>-0.025</v>
+        <v>-0.775</v>
       </c>
       <c r="G49">
         <v>5</v>
@@ -2547,7 +2553,7 @@
         <v>1</v>
       </c>
       <c r="I49" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J49">
         <v>1</v>
@@ -2561,7 +2567,7 @@
     </row>
     <row r="50" spans="1:13">
       <c r="A50" s="1">
-        <v>58</v>
+        <v>217</v>
       </c>
       <c r="B50" t="s">
         <v>14</v>
@@ -2570,28 +2576,28 @@
         <v>63</v>
       </c>
       <c r="D50">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="E50">
-        <v>0.15</v>
+        <v>-0.3</v>
       </c>
       <c r="F50">
-        <v>-0.775</v>
+        <v>-0.75</v>
       </c>
       <c r="G50">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H50">
         <v>1</v>
       </c>
       <c r="I50" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J50">
         <v>1</v>
       </c>
       <c r="L50">
-        <v>1.94</v>
+        <v>1.932</v>
       </c>
       <c r="M50">
         <v>2.655</v>
@@ -2599,7 +2605,7 @@
     </row>
     <row r="51" spans="1:13">
       <c r="A51" s="1">
-        <v>56</v>
+        <v>213</v>
       </c>
       <c r="B51" t="s">
         <v>14</v>
@@ -2608,28 +2614,28 @@
         <v>64</v>
       </c>
       <c r="D51">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="E51">
-        <v>-0.45</v>
+        <v>0.3</v>
       </c>
       <c r="F51">
-        <v>-0.775</v>
+        <v>-0.75</v>
       </c>
       <c r="G51">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H51">
         <v>1</v>
       </c>
       <c r="I51" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J51">
         <v>1</v>
       </c>
       <c r="L51">
-        <v>1.94</v>
+        <v>1.932</v>
       </c>
       <c r="M51">
         <v>2.655</v>
@@ -2637,7 +2643,7 @@
     </row>
     <row r="52" spans="1:13">
       <c r="A52" s="1">
-        <v>55</v>
+        <v>214</v>
       </c>
       <c r="B52" t="s">
         <v>14</v>
@@ -2646,28 +2652,28 @@
         <v>65</v>
       </c>
       <c r="D52">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="E52">
-        <v>-0.9</v>
+        <v>0.3</v>
       </c>
       <c r="F52">
-        <v>-0.025</v>
+        <v>-0.15</v>
       </c>
       <c r="G52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H52">
         <v>1</v>
       </c>
       <c r="I52" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J52">
         <v>1</v>
       </c>
       <c r="L52">
-        <v>1.94</v>
+        <v>1.932</v>
       </c>
       <c r="M52">
         <v>2.655</v>
@@ -2675,7 +2681,7 @@
     </row>
     <row r="53" spans="1:13">
       <c r="A53" s="1">
-        <v>57</v>
+        <v>215</v>
       </c>
       <c r="B53" t="s">
         <v>14</v>
@@ -2684,28 +2690,28 @@
         <v>66</v>
       </c>
       <c r="D53">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="E53">
-        <v>-0.45</v>
+        <v>0.3</v>
       </c>
       <c r="F53">
-        <v>-0.025</v>
+        <v>0.45</v>
       </c>
       <c r="G53">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H53">
         <v>1</v>
       </c>
       <c r="I53" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J53">
         <v>1</v>
       </c>
       <c r="L53">
-        <v>1.94</v>
+        <v>1.932</v>
       </c>
       <c r="M53">
         <v>2.655</v>
@@ -2713,7 +2719,7 @@
     </row>
     <row r="54" spans="1:13">
       <c r="A54" s="1">
-        <v>59</v>
+        <v>216</v>
       </c>
       <c r="B54" t="s">
         <v>14</v>
@@ -2722,28 +2728,28 @@
         <v>67</v>
       </c>
       <c r="D54">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="E54">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="F54">
-        <v>-0.025</v>
+        <v>1.05</v>
       </c>
       <c r="G54">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H54">
         <v>1</v>
       </c>
       <c r="I54" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J54">
         <v>1</v>
       </c>
       <c r="L54">
-        <v>1.94</v>
+        <v>1.932</v>
       </c>
       <c r="M54">
         <v>2.655</v>
@@ -2751,7 +2757,7 @@
     </row>
     <row r="55" spans="1:13">
       <c r="A55" s="1">
-        <v>54</v>
+        <v>220</v>
       </c>
       <c r="B55" t="s">
         <v>14</v>
@@ -2760,28 +2766,28 @@
         <v>68</v>
       </c>
       <c r="D55">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="E55">
-        <v>-0.9</v>
+        <v>-0.3</v>
       </c>
       <c r="F55">
-        <v>-0.775</v>
+        <v>1.05</v>
       </c>
       <c r="G55">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H55">
         <v>1</v>
       </c>
       <c r="I55" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J55">
         <v>1</v>
       </c>
       <c r="L55">
-        <v>1.94</v>
+        <v>1.932</v>
       </c>
       <c r="M55">
         <v>2.655</v>
@@ -2789,7 +2795,7 @@
     </row>
     <row r="56" spans="1:13">
       <c r="A56" s="1">
-        <v>62</v>
+        <v>218</v>
       </c>
       <c r="B56" t="s">
         <v>14</v>
@@ -2804,7 +2810,7 @@
         <v>-0.3</v>
       </c>
       <c r="F56">
-        <v>-0.75</v>
+        <v>-0.15</v>
       </c>
       <c r="G56">
         <v>6</v>
@@ -2813,7 +2819,7 @@
         <v>1</v>
       </c>
       <c r="I56" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J56">
         <v>1</v>
@@ -2827,7 +2833,7 @@
     </row>
     <row r="57" spans="1:13">
       <c r="A57" s="1">
-        <v>63</v>
+        <v>219</v>
       </c>
       <c r="B57" t="s">
         <v>14</v>
@@ -2842,7 +2848,7 @@
         <v>-0.3</v>
       </c>
       <c r="F57">
-        <v>-0.15</v>
+        <v>0.45</v>
       </c>
       <c r="G57">
         <v>6</v>
@@ -2851,7 +2857,7 @@
         <v>1</v>
       </c>
       <c r="I57" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J57">
         <v>1</v>
@@ -2865,7 +2871,7 @@
     </row>
     <row r="58" spans="1:13">
       <c r="A58" s="1">
-        <v>64</v>
+        <v>230</v>
       </c>
       <c r="B58" t="s">
         <v>14</v>
@@ -2874,36 +2880,36 @@
         <v>71</v>
       </c>
       <c r="D58">
-        <v>0</v>
+        <v>0.72</v>
       </c>
       <c r="E58">
-        <v>-0.3</v>
+        <v>0.45</v>
       </c>
       <c r="F58">
-        <v>0.45</v>
-      </c>
-      <c r="G58">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="G58" t="s">
+        <v>91</v>
       </c>
       <c r="H58">
         <v>1</v>
       </c>
       <c r="I58" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J58">
         <v>1</v>
       </c>
       <c r="L58">
+        <v>2.9</v>
+      </c>
+      <c r="M58">
         <v>1.932</v>
-      </c>
-      <c r="M58">
-        <v>2.655</v>
       </c>
     </row>
     <row r="59" spans="1:13">
       <c r="A59" s="1">
-        <v>65</v>
+        <v>231</v>
       </c>
       <c r="B59" t="s">
         <v>14</v>
@@ -2912,36 +2918,36 @@
         <v>72</v>
       </c>
       <c r="D59">
-        <v>0</v>
+        <v>0.72</v>
       </c>
       <c r="E59">
-        <v>-0.3</v>
+        <v>0.6</v>
       </c>
       <c r="F59">
-        <v>1.05</v>
-      </c>
-      <c r="G59">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="G59" t="s">
+        <v>91</v>
       </c>
       <c r="H59">
         <v>1</v>
       </c>
       <c r="I59" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J59">
         <v>1</v>
       </c>
       <c r="L59">
+        <v>2.9</v>
+      </c>
+      <c r="M59">
         <v>1.932</v>
-      </c>
-      <c r="M59">
-        <v>2.655</v>
       </c>
     </row>
     <row r="60" spans="1:13">
       <c r="A60" s="1">
-        <v>66</v>
+        <v>232</v>
       </c>
       <c r="B60" t="s">
         <v>14</v>
@@ -2950,36 +2956,36 @@
         <v>73</v>
       </c>
       <c r="D60">
-        <v>0</v>
+        <v>0.72</v>
       </c>
       <c r="E60">
-        <v>0.3</v>
+        <v>0.75</v>
       </c>
       <c r="F60">
-        <v>-0.75</v>
-      </c>
-      <c r="G60">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="G60" t="s">
+        <v>91</v>
       </c>
       <c r="H60">
         <v>1</v>
       </c>
       <c r="I60" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J60">
         <v>1</v>
       </c>
       <c r="L60">
+        <v>2.9</v>
+      </c>
+      <c r="M60">
         <v>1.932</v>
-      </c>
-      <c r="M60">
-        <v>2.655</v>
       </c>
     </row>
     <row r="61" spans="1:13">
       <c r="A61" s="1">
-        <v>67</v>
+        <v>233</v>
       </c>
       <c r="B61" t="s">
         <v>14</v>
@@ -2988,36 +2994,36 @@
         <v>74</v>
       </c>
       <c r="D61">
-        <v>0</v>
+        <v>0.72</v>
       </c>
       <c r="E61">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="F61">
-        <v>-0.15</v>
-      </c>
-      <c r="G61">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="G61" t="s">
+        <v>91</v>
       </c>
       <c r="H61">
         <v>1</v>
       </c>
       <c r="I61" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J61">
         <v>1</v>
       </c>
       <c r="L61">
+        <v>2.9</v>
+      </c>
+      <c r="M61">
         <v>1.932</v>
-      </c>
-      <c r="M61">
-        <v>2.655</v>
       </c>
     </row>
     <row r="62" spans="1:13">
       <c r="A62" s="1">
-        <v>68</v>
+        <v>234</v>
       </c>
       <c r="B62" t="s">
         <v>14</v>
@@ -3026,36 +3032,36 @@
         <v>75</v>
       </c>
       <c r="D62">
-        <v>0</v>
+        <v>0.72</v>
       </c>
       <c r="E62">
-        <v>0.3</v>
+        <v>1.05</v>
       </c>
       <c r="F62">
-        <v>0.45</v>
-      </c>
-      <c r="G62">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="G62" t="s">
+        <v>91</v>
       </c>
       <c r="H62">
         <v>1</v>
       </c>
       <c r="I62" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J62">
         <v>1</v>
       </c>
       <c r="L62">
+        <v>2.9</v>
+      </c>
+      <c r="M62">
         <v>1.932</v>
-      </c>
-      <c r="M62">
-        <v>2.655</v>
       </c>
     </row>
     <row r="63" spans="1:13">
       <c r="A63" s="1">
-        <v>69</v>
+        <v>235</v>
       </c>
       <c r="B63" t="s">
         <v>14</v>
@@ -3064,36 +3070,36 @@
         <v>76</v>
       </c>
       <c r="D63">
-        <v>0</v>
+        <v>1.41</v>
       </c>
       <c r="E63">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="F63">
-        <v>1.05</v>
-      </c>
-      <c r="G63">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="G63" t="s">
+        <v>91</v>
       </c>
       <c r="H63">
         <v>1</v>
       </c>
       <c r="I63" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J63">
         <v>1</v>
       </c>
       <c r="L63">
+        <v>2.9</v>
+      </c>
+      <c r="M63">
         <v>1.932</v>
-      </c>
-      <c r="M63">
-        <v>2.655</v>
       </c>
     </row>
     <row r="64" spans="1:13">
       <c r="A64" s="1">
-        <v>81</v>
+        <v>236</v>
       </c>
       <c r="B64" t="s">
         <v>14</v>
@@ -3102,22 +3108,22 @@
         <v>77</v>
       </c>
       <c r="D64">
-        <v>0.72</v>
+        <v>1.41</v>
       </c>
       <c r="E64">
-        <v>1.05</v>
+        <v>1.2</v>
       </c>
       <c r="F64">
-        <v>-0.025</v>
+        <v>0</v>
       </c>
       <c r="G64" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H64">
         <v>1</v>
       </c>
       <c r="I64" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J64">
         <v>1</v>
@@ -3131,7 +3137,7 @@
     </row>
     <row r="65" spans="1:13">
       <c r="A65" s="1">
-        <v>76</v>
+        <v>237</v>
       </c>
       <c r="B65" t="s">
         <v>14</v>
@@ -3140,22 +3146,22 @@
         <v>78</v>
       </c>
       <c r="D65">
-        <v>0.12</v>
+        <v>2.01</v>
       </c>
       <c r="E65">
-        <v>1.05</v>
+        <v>0.6</v>
       </c>
       <c r="F65">
-        <v>-0.025</v>
+        <v>0</v>
       </c>
       <c r="G65" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H65">
         <v>1</v>
       </c>
       <c r="I65" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J65">
         <v>1</v>
@@ -3169,7 +3175,7 @@
     </row>
     <row r="66" spans="1:13">
       <c r="A66" s="1">
-        <v>79</v>
+        <v>229</v>
       </c>
       <c r="B66" t="s">
         <v>14</v>
@@ -3181,19 +3187,19 @@
         <v>0.72</v>
       </c>
       <c r="E66">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="F66">
-        <v>-0.025</v>
+        <v>0</v>
       </c>
       <c r="G66" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H66">
         <v>1</v>
       </c>
       <c r="I66" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J66">
         <v>1</v>
@@ -3207,7 +3213,7 @@
     </row>
     <row r="67" spans="1:13">
       <c r="A67" s="1">
-        <v>78</v>
+        <v>238</v>
       </c>
       <c r="B67" t="s">
         <v>14</v>
@@ -3216,22 +3222,22 @@
         <v>80</v>
       </c>
       <c r="D67">
-        <v>0.12</v>
+        <v>2.01</v>
       </c>
       <c r="E67">
-        <v>0.15</v>
+        <v>1.2</v>
       </c>
       <c r="F67">
-        <v>-0.025</v>
+        <v>0</v>
       </c>
       <c r="G67" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H67">
         <v>1</v>
       </c>
       <c r="I67" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J67">
         <v>1</v>
@@ -3245,7 +3251,7 @@
     </row>
     <row r="68" spans="1:13">
       <c r="A68" s="1">
-        <v>77</v>
+        <v>228</v>
       </c>
       <c r="B68" t="s">
         <v>14</v>
@@ -3254,22 +3260,22 @@
         <v>81</v>
       </c>
       <c r="D68">
-        <v>0.12</v>
+        <v>0.72</v>
       </c>
       <c r="E68">
-        <v>0.6</v>
+        <v>0.15</v>
       </c>
       <c r="F68">
-        <v>-0.025</v>
+        <v>0</v>
       </c>
       <c r="G68" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H68">
         <v>1</v>
       </c>
       <c r="I68" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J68">
         <v>1</v>
@@ -3283,7 +3289,7 @@
     </row>
     <row r="69" spans="1:13">
       <c r="A69" s="1">
-        <v>75</v>
+        <v>226</v>
       </c>
       <c r="B69" t="s">
         <v>14</v>
@@ -3292,22 +3298,22 @@
         <v>82</v>
       </c>
       <c r="D69">
-        <v>2.31</v>
+        <v>0.12</v>
       </c>
       <c r="E69">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="F69">
-        <v>-0.025</v>
+        <v>0</v>
       </c>
       <c r="G69" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H69">
         <v>1</v>
       </c>
       <c r="I69" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J69">
         <v>1</v>
@@ -3321,7 +3327,7 @@
     </row>
     <row r="70" spans="1:13">
       <c r="A70" s="1">
-        <v>74</v>
+        <v>225</v>
       </c>
       <c r="B70" t="s">
         <v>14</v>
@@ -3330,22 +3336,22 @@
         <v>83</v>
       </c>
       <c r="D70">
-        <v>2.31</v>
+        <v>0.12</v>
       </c>
       <c r="E70">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="F70">
-        <v>-0.025</v>
+        <v>0</v>
       </c>
       <c r="G70" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H70">
         <v>1</v>
       </c>
       <c r="I70" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J70">
         <v>1</v>
@@ -3359,7 +3365,7 @@
     </row>
     <row r="71" spans="1:13">
       <c r="A71" s="1">
-        <v>73</v>
+        <v>224</v>
       </c>
       <c r="B71" t="s">
         <v>14</v>
@@ -3368,22 +3374,22 @@
         <v>84</v>
       </c>
       <c r="D71">
-        <v>2.31</v>
+        <v>0.12</v>
       </c>
       <c r="E71">
-        <v>0.15</v>
+        <v>0.6</v>
       </c>
       <c r="F71">
-        <v>-0.025</v>
+        <v>0</v>
       </c>
       <c r="G71" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H71">
         <v>1</v>
       </c>
       <c r="I71" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J71">
         <v>1</v>
@@ -3397,7 +3403,7 @@
     </row>
     <row r="72" spans="1:13">
       <c r="A72" s="1">
-        <v>71</v>
+        <v>223</v>
       </c>
       <c r="B72" t="s">
         <v>14</v>
@@ -3406,22 +3412,22 @@
         <v>85</v>
       </c>
       <c r="D72">
-        <v>1.41</v>
+        <v>0.12</v>
       </c>
       <c r="E72">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="F72">
-        <v>-0.025</v>
+        <v>0</v>
       </c>
       <c r="G72" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H72">
         <v>1</v>
       </c>
       <c r="I72" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J72">
         <v>1</v>
@@ -3435,7 +3441,7 @@
     </row>
     <row r="73" spans="1:13">
       <c r="A73" s="1">
-        <v>70</v>
+        <v>222</v>
       </c>
       <c r="B73" t="s">
         <v>14</v>
@@ -3444,22 +3450,22 @@
         <v>86</v>
       </c>
       <c r="D73">
-        <v>1.41</v>
+        <v>0.12</v>
       </c>
       <c r="E73">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="F73">
-        <v>-0.025</v>
+        <v>0</v>
       </c>
       <c r="G73" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H73">
         <v>1</v>
       </c>
       <c r="I73" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J73">
         <v>1</v>
@@ -3473,7 +3479,7 @@
     </row>
     <row r="74" spans="1:13">
       <c r="A74" s="1">
-        <v>80</v>
+        <v>221</v>
       </c>
       <c r="B74" t="s">
         <v>14</v>
@@ -3482,22 +3488,22 @@
         <v>87</v>
       </c>
       <c r="D74">
-        <v>0.72</v>
+        <v>0.12</v>
       </c>
       <c r="E74">
-        <v>0.6</v>
+        <v>0.15</v>
       </c>
       <c r="F74">
-        <v>-0.025</v>
+        <v>0</v>
       </c>
       <c r="G74" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H74">
         <v>1</v>
       </c>
       <c r="I74" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J74">
         <v>1</v>
@@ -3511,7 +3517,7 @@
     </row>
     <row r="75" spans="1:13">
       <c r="A75" s="1">
-        <v>72</v>
+        <v>239</v>
       </c>
       <c r="B75" t="s">
         <v>14</v>
@@ -3520,30 +3526,106 @@
         <v>88</v>
       </c>
       <c r="D75">
-        <v>1.41</v>
+        <v>2.61</v>
       </c>
       <c r="E75">
+        <v>0.6</v>
+      </c>
+      <c r="F75">
+        <v>0</v>
+      </c>
+      <c r="G75" t="s">
+        <v>91</v>
+      </c>
+      <c r="H75">
+        <v>1</v>
+      </c>
+      <c r="I75" t="s">
+        <v>93</v>
+      </c>
+      <c r="J75">
+        <v>1</v>
+      </c>
+      <c r="L75">
+        <v>2.9</v>
+      </c>
+      <c r="M75">
+        <v>1.932</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13">
+      <c r="A76" s="1">
+        <v>227</v>
+      </c>
+      <c r="B76" t="s">
+        <v>14</v>
+      </c>
+      <c r="C76" t="s">
+        <v>89</v>
+      </c>
+      <c r="D76">
+        <v>0.12</v>
+      </c>
+      <c r="E76">
+        <v>1.05</v>
+      </c>
+      <c r="F76">
+        <v>0</v>
+      </c>
+      <c r="G76" t="s">
+        <v>91</v>
+      </c>
+      <c r="H76">
+        <v>1</v>
+      </c>
+      <c r="I76" t="s">
+        <v>93</v>
+      </c>
+      <c r="J76">
+        <v>1</v>
+      </c>
+      <c r="L76">
+        <v>2.9</v>
+      </c>
+      <c r="M76">
+        <v>1.932</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13">
+      <c r="A77" s="1">
+        <v>240</v>
+      </c>
+      <c r="B77" t="s">
+        <v>14</v>
+      </c>
+      <c r="C77" t="s">
+        <v>90</v>
+      </c>
+      <c r="D77">
+        <v>2.61</v>
+      </c>
+      <c r="E77">
         <v>1.2</v>
       </c>
-      <c r="F75">
-        <v>-0.025</v>
-      </c>
-      <c r="G75" t="s">
-        <v>89</v>
-      </c>
-      <c r="H75">
-        <v>1</v>
-      </c>
-      <c r="I75" t="s">
+      <c r="F77">
+        <v>0</v>
+      </c>
+      <c r="G77" t="s">
         <v>91</v>
       </c>
-      <c r="J75">
-        <v>1</v>
-      </c>
-      <c r="L75">
-        <v>2.9</v>
-      </c>
-      <c r="M75">
+      <c r="H77">
+        <v>1</v>
+      </c>
+      <c r="I77" t="s">
+        <v>93</v>
+      </c>
+      <c r="J77">
+        <v>1</v>
+      </c>
+      <c r="L77">
+        <v>2.9</v>
+      </c>
+      <c r="M77">
         <v>1.932</v>
       </c>
     </row>
@@ -3603,31 +3685,31 @@
     </row>
     <row r="2" spans="1:15">
       <c r="A2" s="1">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D2">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="E2">
-        <v>0.21</v>
+        <v>0.023</v>
       </c>
       <c r="F2">
-        <v>-0.05</v>
+        <v>0.387</v>
       </c>
       <c r="G2">
         <v>3</v>
       </c>
-      <c r="H2">
-        <v>6</v>
+      <c r="H2" t="s">
+        <v>103</v>
       </c>
       <c r="I2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -3641,31 +3723,31 @@
     </row>
     <row r="3" spans="1:15">
       <c r="A3" s="1">
-        <v>237</v>
+        <v>94</v>
       </c>
       <c r="B3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D3">
-        <v>1.202</v>
+        <v>0.6</v>
       </c>
       <c r="E3">
-        <v>0.16</v>
+        <v>0.21</v>
       </c>
       <c r="F3">
-        <v>-0.181</v>
+        <v>-0.05</v>
       </c>
       <c r="G3">
         <v>3</v>
       </c>
-      <c r="H3">
-        <v>6</v>
+      <c r="H3" t="s">
+        <v>103</v>
       </c>
       <c r="I3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -3679,16 +3761,16 @@
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="1">
-        <v>238</v>
+        <v>164</v>
       </c>
       <c r="B4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D4">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -3699,11 +3781,11 @@
       <c r="G4">
         <v>5</v>
       </c>
-      <c r="H4">
-        <v>6</v>
+      <c r="H4" t="s">
+        <v>103</v>
       </c>
       <c r="I4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -3717,13 +3799,13 @@
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="1">
-        <v>114</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D5">
         <v>2.31</v>
@@ -3735,13 +3817,13 @@
         <v>0.547</v>
       </c>
       <c r="G5" t="s">
-        <v>89</v>
-      </c>
-      <c r="H5">
-        <v>6</v>
+        <v>91</v>
+      </c>
+      <c r="H5" t="s">
+        <v>103</v>
       </c>
       <c r="I5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -3755,13 +3837,13 @@
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="1">
-        <v>235</v>
+        <v>161</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D6">
         <v>1.285</v>
@@ -3773,13 +3855,13 @@
         <v>-0.024</v>
       </c>
       <c r="G6" t="s">
-        <v>89</v>
-      </c>
-      <c r="H6">
-        <v>6</v>
+        <v>91</v>
+      </c>
+      <c r="H6" t="s">
+        <v>103</v>
       </c>
       <c r="I6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -3793,31 +3875,31 @@
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="1">
-        <v>231</v>
+        <v>159</v>
       </c>
       <c r="B7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D7">
-        <v>2.31</v>
+        <v>1.41</v>
       </c>
       <c r="E7">
-        <v>1.74</v>
+        <v>1.692</v>
       </c>
       <c r="F7">
         <v>0.825</v>
       </c>
       <c r="G7" t="s">
-        <v>89</v>
-      </c>
-      <c r="H7">
-        <v>6</v>
+        <v>91</v>
+      </c>
+      <c r="H7" t="s">
+        <v>103</v>
       </c>
       <c r="I7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -3831,31 +3913,31 @@
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="1">
-        <v>233</v>
+        <v>157</v>
       </c>
       <c r="B8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D8">
-        <v>1.41</v>
+        <v>2.31</v>
       </c>
       <c r="E8">
-        <v>1.692</v>
+        <v>1.74</v>
       </c>
       <c r="F8">
         <v>0.825</v>
       </c>
       <c r="G8" t="s">
-        <v>89</v>
-      </c>
-      <c r="H8">
-        <v>6</v>
+        <v>91</v>
+      </c>
+      <c r="H8" t="s">
+        <v>103</v>
       </c>
       <c r="I8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -3869,13 +3951,13 @@
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="1">
-        <v>230</v>
+        <v>156</v>
       </c>
       <c r="B9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C9" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D9">
         <v>1.06</v>
@@ -3887,13 +3969,13 @@
         <v>0.275</v>
       </c>
       <c r="G9" t="s">
-        <v>89</v>
-      </c>
-      <c r="H9">
-        <v>6</v>
+        <v>91</v>
+      </c>
+      <c r="H9" t="s">
+        <v>103</v>
       </c>
       <c r="I9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J9">
         <v>1</v>
@@ -3923,13 +4005,13 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
tmp for countplusy and countminusy
</commit_message>
<xml_diff>
--- a/Greyform/Python_Application/exporteddatassss(with TMP)(draft)(tetra).xlsx
+++ b/Greyform/Python_Application/exporteddatassss(with TMP)(draft)(tetra).xlsx
@@ -1,28 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MokZhiZhuan\OneDrive - WINSYS TECHNOLOGY PTE LTD\Documents\GitHub\GreyForm_UI\Greyform\Python_Application\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACAE0D87-4419-4FE4-863D-5B1C23EEFF82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Stage 2" sheetId="1" r:id="rId1"/>
     <sheet name="Stage 3" sheetId="2" r:id="rId2"/>
     <sheet name="Obstacles" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="144">
   <si>
     <t>Marking type</t>
   </si>
@@ -285,6 +279,9 @@
     <t>F</t>
   </si>
   <si>
+    <t>+</t>
+  </si>
+  <si>
     <t>blank</t>
   </si>
   <si>
@@ -433,6 +430,9 @@
   </si>
   <si>
     <t>BSS.FLOOR DRAIN_150:BSS.FLOOR DRAIN_150:1091065</t>
+  </si>
+  <si>
+    <t>6</t>
   </si>
   <si>
     <t>Point number/name</t>
@@ -453,8 +453,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -517,21 +517,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -569,7 +561,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -603,7 +595,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -638,10 +629,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -814,25 +804,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O72"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.28515625" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -876,7 +852,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15">
       <c r="A2" s="1">
         <v>182</v>
       </c>
@@ -893,7 +869,7 @@
         <v>-1.35</v>
       </c>
       <c r="F2">
-        <v>-0.17499999999999999</v>
+        <v>-0.175</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -902,7 +878,7 @@
         <v>1</v>
       </c>
       <c r="I2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -911,10 +887,10 @@
         <v>2.76</v>
       </c>
       <c r="M2">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
       <c r="A3" s="1">
         <v>181</v>
       </c>
@@ -931,7 +907,7 @@
         <v>-1.35</v>
       </c>
       <c r="F3">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -940,7 +916,7 @@
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -949,10 +925,10 @@
         <v>2.76</v>
       </c>
       <c r="M3">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
       <c r="A4" s="1">
         <v>180</v>
       </c>
@@ -969,7 +945,7 @@
         <v>-0.35</v>
       </c>
       <c r="F4">
-        <v>1.0249999999999999</v>
+        <v>1.025</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -978,7 +954,7 @@
         <v>1</v>
       </c>
       <c r="I4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -987,10 +963,10 @@
         <v>2.76</v>
       </c>
       <c r="M4">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
       <c r="A5" s="1">
         <v>179</v>
       </c>
@@ -1007,7 +983,7 @@
         <v>-0.35</v>
       </c>
       <c r="F5">
-        <v>0.42499999999999999</v>
+        <v>0.425</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -1016,7 +992,7 @@
         <v>1</v>
       </c>
       <c r="I5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -1025,10 +1001,10 @@
         <v>2.76</v>
       </c>
       <c r="M5">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6" s="1">
         <v>178</v>
       </c>
@@ -1045,7 +1021,7 @@
         <v>-0.35</v>
       </c>
       <c r="F6">
-        <v>-0.17499999999999999</v>
+        <v>-0.175</v>
       </c>
       <c r="G6">
         <v>1</v>
@@ -1054,7 +1030,7 @@
         <v>1</v>
       </c>
       <c r="I6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -1063,10 +1039,10 @@
         <v>2.76</v>
       </c>
       <c r="M6">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
       <c r="A7" s="1">
         <v>177</v>
       </c>
@@ -1083,7 +1059,7 @@
         <v>-0.35</v>
       </c>
       <c r="F7">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G7">
         <v>1</v>
@@ -1092,7 +1068,7 @@
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -1101,10 +1077,10 @@
         <v>2.76</v>
       </c>
       <c r="M7">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8" s="1">
         <v>176</v>
       </c>
@@ -1121,7 +1097,7 @@
         <v>-0.03</v>
       </c>
       <c r="F8">
-        <v>1.0249999999999999</v>
+        <v>1.025</v>
       </c>
       <c r="G8">
         <v>1</v>
@@ -1130,7 +1106,7 @@
         <v>1</v>
       </c>
       <c r="I8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -1139,10 +1115,10 @@
         <v>2.76</v>
       </c>
       <c r="M8">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
       <c r="A9" s="1">
         <v>175</v>
       </c>
@@ -1159,7 +1135,7 @@
         <v>-0.03</v>
       </c>
       <c r="F9">
-        <v>0.42499999999999999</v>
+        <v>0.425</v>
       </c>
       <c r="G9">
         <v>1</v>
@@ -1168,7 +1144,7 @@
         <v>1</v>
       </c>
       <c r="I9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J9">
         <v>1</v>
@@ -1177,10 +1153,10 @@
         <v>2.76</v>
       </c>
       <c r="M9">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10" s="1">
         <v>174</v>
       </c>
@@ -1197,7 +1173,7 @@
         <v>-0.03</v>
       </c>
       <c r="F10">
-        <v>-0.17499999999999999</v>
+        <v>-0.175</v>
       </c>
       <c r="G10">
         <v>1</v>
@@ -1206,7 +1182,7 @@
         <v>1</v>
       </c>
       <c r="I10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J10">
         <v>1</v>
@@ -1215,10 +1191,10 @@
         <v>2.76</v>
       </c>
       <c r="M10">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
       <c r="A11" s="1">
         <v>173</v>
       </c>
@@ -1235,7 +1211,7 @@
         <v>-0.03</v>
       </c>
       <c r="F11">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G11">
         <v>1</v>
@@ -1244,7 +1220,7 @@
         <v>1</v>
       </c>
       <c r="I11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J11">
         <v>1</v>
@@ -1253,10 +1229,10 @@
         <v>2.76</v>
       </c>
       <c r="M11">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
       <c r="A12" s="1">
         <v>172</v>
       </c>
@@ -1273,7 +1249,7 @@
         <v>0.47</v>
       </c>
       <c r="F12">
-        <v>1.0249999999999999</v>
+        <v>1.025</v>
       </c>
       <c r="G12">
         <v>1</v>
@@ -1282,7 +1258,7 @@
         <v>1</v>
       </c>
       <c r="I12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J12">
         <v>1</v>
@@ -1291,10 +1267,10 @@
         <v>2.76</v>
       </c>
       <c r="M12">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
       <c r="A13" s="1">
         <v>171</v>
       </c>
@@ -1311,7 +1287,7 @@
         <v>0.47</v>
       </c>
       <c r="F13">
-        <v>0.42499999999999999</v>
+        <v>0.425</v>
       </c>
       <c r="G13">
         <v>1</v>
@@ -1320,7 +1296,7 @@
         <v>1</v>
       </c>
       <c r="I13" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J13">
         <v>1</v>
@@ -1329,10 +1305,10 @@
         <v>2.76</v>
       </c>
       <c r="M13">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
       <c r="A14" s="1">
         <v>170</v>
       </c>
@@ -1349,7 +1325,7 @@
         <v>0.47</v>
       </c>
       <c r="F14">
-        <v>-0.17499999999999999</v>
+        <v>-0.175</v>
       </c>
       <c r="G14">
         <v>1</v>
@@ -1358,7 +1334,7 @@
         <v>1</v>
       </c>
       <c r="I14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J14">
         <v>1</v>
@@ -1367,10 +1343,10 @@
         <v>2.76</v>
       </c>
       <c r="M14">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
       <c r="A15" s="1">
         <v>169</v>
       </c>
@@ -1387,7 +1363,7 @@
         <v>0.47</v>
       </c>
       <c r="F15">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G15">
         <v>1</v>
@@ -1396,7 +1372,7 @@
         <v>1</v>
       </c>
       <c r="I15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J15">
         <v>1</v>
@@ -1405,10 +1381,10 @@
         <v>2.76</v>
       </c>
       <c r="M15">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
       <c r="A16" s="1">
         <v>168</v>
       </c>
@@ -1425,7 +1401,7 @@
         <v>0.49</v>
       </c>
       <c r="F16">
-        <v>1.0249999999999999</v>
+        <v>1.025</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -1434,7 +1410,7 @@
         <v>1</v>
       </c>
       <c r="I16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J16">
         <v>1</v>
@@ -1443,10 +1419,10 @@
         <v>2.76</v>
       </c>
       <c r="M16">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17" s="1">
         <v>167</v>
       </c>
@@ -1463,7 +1439,7 @@
         <v>0.49</v>
       </c>
       <c r="F17">
-        <v>0.42499999999999999</v>
+        <v>0.425</v>
       </c>
       <c r="G17">
         <v>1</v>
@@ -1472,7 +1448,7 @@
         <v>1</v>
       </c>
       <c r="I17" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J17">
         <v>1</v>
@@ -1481,10 +1457,10 @@
         <v>2.76</v>
       </c>
       <c r="M17">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
       <c r="A18" s="1">
         <v>166</v>
       </c>
@@ -1501,7 +1477,7 @@
         <v>0.49</v>
       </c>
       <c r="F18">
-        <v>-0.17499999999999999</v>
+        <v>-0.175</v>
       </c>
       <c r="G18">
         <v>1</v>
@@ -1510,7 +1486,7 @@
         <v>1</v>
       </c>
       <c r="I18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J18">
         <v>1</v>
@@ -1519,10 +1495,10 @@
         <v>2.76</v>
       </c>
       <c r="M18">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
       <c r="A19" s="1">
         <v>165</v>
       </c>
@@ -1539,7 +1515,7 @@
         <v>0.49</v>
       </c>
       <c r="F19">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -1548,7 +1524,7 @@
         <v>1</v>
       </c>
       <c r="I19" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J19">
         <v>1</v>
@@ -1557,10 +1533,10 @@
         <v>2.76</v>
       </c>
       <c r="M19">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
       <c r="A20" s="1">
         <v>164</v>
       </c>
@@ -1574,10 +1550,10 @@
         <v>0</v>
       </c>
       <c r="E20">
-        <v>0.93500000000000005</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F20">
-        <v>1.0249999999999999</v>
+        <v>1.025</v>
       </c>
       <c r="G20">
         <v>1</v>
@@ -1586,7 +1562,7 @@
         <v>1</v>
       </c>
       <c r="I20" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J20">
         <v>1</v>
@@ -1595,10 +1571,10 @@
         <v>2.76</v>
       </c>
       <c r="M20">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
       <c r="A21" s="1">
         <v>163</v>
       </c>
@@ -1612,10 +1588,10 @@
         <v>0</v>
       </c>
       <c r="E21">
-        <v>0.93500000000000005</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F21">
-        <v>0.42499999999999999</v>
+        <v>0.425</v>
       </c>
       <c r="G21">
         <v>1</v>
@@ -1624,7 +1600,7 @@
         <v>1</v>
       </c>
       <c r="I21" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J21">
         <v>1</v>
@@ -1633,10 +1609,10 @@
         <v>2.76</v>
       </c>
       <c r="M21">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
       <c r="A22" s="1">
         <v>162</v>
       </c>
@@ -1650,10 +1626,10 @@
         <v>0</v>
       </c>
       <c r="E22">
-        <v>0.93500000000000005</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F22">
-        <v>-0.17499999999999999</v>
+        <v>-0.175</v>
       </c>
       <c r="G22">
         <v>1</v>
@@ -1662,7 +1638,7 @@
         <v>1</v>
       </c>
       <c r="I22" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J22">
         <v>1</v>
@@ -1671,10 +1647,10 @@
         <v>2.76</v>
       </c>
       <c r="M22">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13">
       <c r="A23" s="1">
         <v>161</v>
       </c>
@@ -1688,10 +1664,10 @@
         <v>0</v>
       </c>
       <c r="E23">
-        <v>0.93500000000000005</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F23">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G23">
         <v>1</v>
@@ -1700,7 +1676,7 @@
         <v>1</v>
       </c>
       <c r="I23" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J23">
         <v>1</v>
@@ -1709,10 +1685,10 @@
         <v>2.76</v>
       </c>
       <c r="M23">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
       <c r="A24" s="1">
         <v>183</v>
       </c>
@@ -1729,7 +1705,7 @@
         <v>-1.35</v>
       </c>
       <c r="F24">
-        <v>0.42499999999999999</v>
+        <v>0.425</v>
       </c>
       <c r="G24">
         <v>1</v>
@@ -1738,7 +1714,7 @@
         <v>1</v>
       </c>
       <c r="I24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J24">
         <v>1</v>
@@ -1747,10 +1723,10 @@
         <v>2.76</v>
       </c>
       <c r="M24">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13">
       <c r="A25" s="1">
         <v>184</v>
       </c>
@@ -1767,7 +1743,7 @@
         <v>-1.35</v>
       </c>
       <c r="F25">
-        <v>1.0249999999999999</v>
+        <v>1.025</v>
       </c>
       <c r="G25">
         <v>1</v>
@@ -1776,7 +1752,7 @@
         <v>1</v>
       </c>
       <c r="I25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J25">
         <v>1</v>
@@ -1785,10 +1761,10 @@
         <v>2.76</v>
       </c>
       <c r="M25">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13">
       <c r="A26" s="1">
         <v>185</v>
       </c>
@@ -1814,7 +1790,7 @@
         <v>1</v>
       </c>
       <c r="I26" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J26">
         <v>1</v>
@@ -1823,10 +1799,10 @@
         <v>1.2</v>
       </c>
       <c r="M26">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
       <c r="A27" s="1">
         <v>186</v>
       </c>
@@ -1852,7 +1828,7 @@
         <v>1</v>
       </c>
       <c r="I27" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J27">
         <v>1</v>
@@ -1861,10 +1837,10 @@
         <v>1.2</v>
       </c>
       <c r="M27">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13">
       <c r="A28" s="1">
         <v>188</v>
       </c>
@@ -1890,7 +1866,7 @@
         <v>1</v>
       </c>
       <c r="I28" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J28">
         <v>1</v>
@@ -1899,10 +1875,10 @@
         <v>1.2</v>
       </c>
       <c r="M28">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
       <c r="A29" s="1">
         <v>187</v>
       </c>
@@ -1928,7 +1904,7 @@
         <v>1</v>
       </c>
       <c r="I29" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J29">
         <v>1</v>
@@ -1937,10 +1913,10 @@
         <v>1.2</v>
       </c>
       <c r="M29">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
       <c r="A30" s="1">
         <v>189</v>
       </c>
@@ -1954,10 +1930,10 @@
         <v>0.6</v>
       </c>
       <c r="E30">
-        <v>-0.93500000000000005</v>
+        <v>-0.9350000000000001</v>
       </c>
       <c r="F30">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G30">
         <v>3</v>
@@ -1966,7 +1942,7 @@
         <v>1</v>
       </c>
       <c r="I30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J30">
         <v>1</v>
@@ -1975,10 +1951,10 @@
         <v>0.96</v>
       </c>
       <c r="M30">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
       <c r="A31" s="1">
         <v>190</v>
       </c>
@@ -1992,10 +1968,10 @@
         <v>0.6</v>
       </c>
       <c r="E31">
-        <v>-0.93500000000000005</v>
+        <v>-0.9350000000000001</v>
       </c>
       <c r="F31">
-        <v>-0.17499999999999999</v>
+        <v>-0.175</v>
       </c>
       <c r="G31">
         <v>3</v>
@@ -2004,7 +1980,7 @@
         <v>1</v>
       </c>
       <c r="I31" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J31">
         <v>1</v>
@@ -2013,10 +1989,10 @@
         <v>0.96</v>
       </c>
       <c r="M31">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13">
       <c r="A32" s="1">
         <v>191</v>
       </c>
@@ -2030,10 +2006,10 @@
         <v>0.6</v>
       </c>
       <c r="E32">
-        <v>-0.93500000000000005</v>
+        <v>-0.9350000000000001</v>
       </c>
       <c r="F32">
-        <v>0.42499999999999999</v>
+        <v>0.425</v>
       </c>
       <c r="G32">
         <v>3</v>
@@ -2042,7 +2018,7 @@
         <v>1</v>
       </c>
       <c r="I32" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J32">
         <v>1</v>
@@ -2051,10 +2027,10 @@
         <v>0.96</v>
       </c>
       <c r="M32">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13">
       <c r="A33" s="1">
         <v>192</v>
       </c>
@@ -2068,10 +2044,10 @@
         <v>0.6</v>
       </c>
       <c r="E33">
-        <v>-0.93500000000000005</v>
+        <v>-0.9350000000000001</v>
       </c>
       <c r="F33">
-        <v>1.0249999999999999</v>
+        <v>1.025</v>
       </c>
       <c r="G33">
         <v>3</v>
@@ -2080,7 +2056,7 @@
         <v>1</v>
       </c>
       <c r="I33" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J33">
         <v>1</v>
@@ -2089,10 +2065,10 @@
         <v>0.96</v>
       </c>
       <c r="M33">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13">
       <c r="A34" s="1">
         <v>196</v>
       </c>
@@ -2109,7 +2085,7 @@
         <v>0.3</v>
       </c>
       <c r="F34">
-        <v>1.0249999999999999</v>
+        <v>1.025</v>
       </c>
       <c r="G34">
         <v>4</v>
@@ -2118,7 +2094,7 @@
         <v>1</v>
       </c>
       <c r="I34" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J34">
         <v>1</v>
@@ -2127,10 +2103,10 @@
         <v>0.6</v>
       </c>
       <c r="M34">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13">
       <c r="A35" s="1">
         <v>195</v>
       </c>
@@ -2147,7 +2123,7 @@
         <v>0.3</v>
       </c>
       <c r="F35">
-        <v>0.42499999999999999</v>
+        <v>0.425</v>
       </c>
       <c r="G35">
         <v>4</v>
@@ -2156,7 +2132,7 @@
         <v>1</v>
       </c>
       <c r="I35" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J35">
         <v>1</v>
@@ -2165,10 +2141,10 @@
         <v>0.6</v>
       </c>
       <c r="M35">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13">
       <c r="A36" s="1">
         <v>194</v>
       </c>
@@ -2185,7 +2161,7 @@
         <v>0.3</v>
       </c>
       <c r="F36">
-        <v>-0.17499999999999999</v>
+        <v>-0.175</v>
       </c>
       <c r="G36">
         <v>4</v>
@@ -2194,7 +2170,7 @@
         <v>1</v>
       </c>
       <c r="I36" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J36">
         <v>1</v>
@@ -2203,10 +2179,10 @@
         <v>0.6</v>
       </c>
       <c r="M36">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
       <c r="A37" s="1">
         <v>193</v>
       </c>
@@ -2223,7 +2199,7 @@
         <v>0.3</v>
       </c>
       <c r="F37">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G37">
         <v>4</v>
@@ -2232,7 +2208,7 @@
         <v>1</v>
       </c>
       <c r="I37" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J37">
         <v>1</v>
@@ -2241,10 +2217,10 @@
         <v>0.6</v>
       </c>
       <c r="M37">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13">
       <c r="A38" s="1">
         <v>197</v>
       </c>
@@ -2261,7 +2237,7 @@
         <v>0.93</v>
       </c>
       <c r="F38">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G38">
         <v>5</v>
@@ -2270,7 +2246,7 @@
         <v>1</v>
       </c>
       <c r="I38" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J38">
         <v>1</v>
@@ -2279,10 +2255,10 @@
         <v>1.8</v>
       </c>
       <c r="M38">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13">
       <c r="A39" s="1">
         <v>198</v>
       </c>
@@ -2299,7 +2275,7 @@
         <v>0.48</v>
       </c>
       <c r="F39">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G39">
         <v>5</v>
@@ -2308,7 +2284,7 @@
         <v>1</v>
       </c>
       <c r="I39" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J39">
         <v>1</v>
@@ -2317,10 +2293,10 @@
         <v>1.8</v>
       </c>
       <c r="M39">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13">
       <c r="A40" s="1">
         <v>199</v>
       </c>
@@ -2337,7 +2313,7 @@
         <v>0.03</v>
       </c>
       <c r="F40">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G40">
         <v>5</v>
@@ -2346,7 +2322,7 @@
         <v>1</v>
       </c>
       <c r="I40" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J40">
         <v>1</v>
@@ -2355,10 +2331,10 @@
         <v>1.8</v>
       </c>
       <c r="M40">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13">
       <c r="A41" s="1">
         <v>200</v>
       </c>
@@ -2375,7 +2351,7 @@
         <v>1.155</v>
       </c>
       <c r="F41">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G41">
         <v>5</v>
@@ -2384,7 +2360,7 @@
         <v>1</v>
       </c>
       <c r="I41" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J41">
         <v>1</v>
@@ -2393,10 +2369,10 @@
         <v>1.8</v>
       </c>
       <c r="M41">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13">
       <c r="A42" s="1">
         <v>201</v>
       </c>
@@ -2413,7 +2389,7 @@
         <v>1.155</v>
       </c>
       <c r="F42">
-        <v>-0.17499999999999999</v>
+        <v>-0.175</v>
       </c>
       <c r="G42">
         <v>5</v>
@@ -2422,7 +2398,7 @@
         <v>1</v>
       </c>
       <c r="I42" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J42">
         <v>1</v>
@@ -2431,10 +2407,10 @@
         <v>1.8</v>
       </c>
       <c r="M42">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13">
       <c r="A43" s="1">
         <v>202</v>
       </c>
@@ -2451,7 +2427,7 @@
         <v>1.155</v>
       </c>
       <c r="F43">
-        <v>0.42499999999999999</v>
+        <v>0.425</v>
       </c>
       <c r="G43">
         <v>5</v>
@@ -2460,7 +2436,7 @@
         <v>1</v>
       </c>
       <c r="I43" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J43">
         <v>1</v>
@@ -2469,10 +2445,10 @@
         <v>1.8</v>
       </c>
       <c r="M43">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13">
       <c r="A44" s="1">
         <v>203</v>
       </c>
@@ -2489,7 +2465,7 @@
         <v>1.155</v>
       </c>
       <c r="F44">
-        <v>1.0249999999999999</v>
+        <v>1.025</v>
       </c>
       <c r="G44">
         <v>5</v>
@@ -2498,7 +2474,7 @@
         <v>1</v>
       </c>
       <c r="I44" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J44">
         <v>1</v>
@@ -2507,10 +2483,10 @@
         <v>1.8</v>
       </c>
       <c r="M44">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13">
       <c r="A45" s="1">
         <v>207</v>
       </c>
@@ -2527,7 +2503,7 @@
         <v>0.3</v>
       </c>
       <c r="F45">
-        <v>1.0249999999999999</v>
+        <v>1.025</v>
       </c>
       <c r="G45">
         <v>6</v>
@@ -2536,7 +2512,7 @@
         <v>1</v>
       </c>
       <c r="I45" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J45">
         <v>1</v>
@@ -2545,10 +2521,10 @@
         <v>1.8</v>
       </c>
       <c r="M45">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13">
       <c r="A46" s="1">
         <v>205</v>
       </c>
@@ -2565,7 +2541,7 @@
         <v>0.3</v>
       </c>
       <c r="F46">
-        <v>-0.17499999999999999</v>
+        <v>-0.175</v>
       </c>
       <c r="G46">
         <v>6</v>
@@ -2574,7 +2550,7 @@
         <v>1</v>
       </c>
       <c r="I46" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J46">
         <v>1</v>
@@ -2583,10 +2559,10 @@
         <v>1.8</v>
       </c>
       <c r="M46">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13">
       <c r="A47" s="1">
         <v>206</v>
       </c>
@@ -2603,7 +2579,7 @@
         <v>0.3</v>
       </c>
       <c r="F47">
-        <v>0.42499999999999999</v>
+        <v>0.425</v>
       </c>
       <c r="G47">
         <v>6</v>
@@ -2612,7 +2588,7 @@
         <v>1</v>
       </c>
       <c r="I47" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J47">
         <v>1</v>
@@ -2621,10 +2597,10 @@
         <v>1.8</v>
       </c>
       <c r="M47">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13">
       <c r="A48" s="1">
         <v>208</v>
       </c>
@@ -2641,7 +2617,7 @@
         <v>-0.3</v>
       </c>
       <c r="F48">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G48">
         <v>6</v>
@@ -2650,7 +2626,7 @@
         <v>1</v>
       </c>
       <c r="I48" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J48">
         <v>1</v>
@@ -2659,10 +2635,10 @@
         <v>1.8</v>
       </c>
       <c r="M48">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13">
       <c r="A49" s="1">
         <v>204</v>
       </c>
@@ -2679,7 +2655,7 @@
         <v>0.3</v>
       </c>
       <c r="F49">
-        <v>-0.77500000000000002</v>
+        <v>-0.775</v>
       </c>
       <c r="G49">
         <v>6</v>
@@ -2688,7 +2664,7 @@
         <v>1</v>
       </c>
       <c r="I49" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J49">
         <v>1</v>
@@ -2697,10 +2673,10 @@
         <v>1.8</v>
       </c>
       <c r="M49">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13">
       <c r="A50" s="1">
         <v>210</v>
       </c>
@@ -2717,7 +2693,7 @@
         <v>-0.3</v>
       </c>
       <c r="F50">
-        <v>0.42499999999999999</v>
+        <v>0.425</v>
       </c>
       <c r="G50">
         <v>6</v>
@@ -2726,7 +2702,7 @@
         <v>1</v>
       </c>
       <c r="I50" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J50">
         <v>1</v>
@@ -2735,10 +2711,10 @@
         <v>1.8</v>
       </c>
       <c r="M50">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13">
       <c r="A51" s="1">
         <v>211</v>
       </c>
@@ -2755,7 +2731,7 @@
         <v>-0.3</v>
       </c>
       <c r="F51">
-        <v>1.0249999999999999</v>
+        <v>1.025</v>
       </c>
       <c r="G51">
         <v>6</v>
@@ -2764,7 +2740,7 @@
         <v>1</v>
       </c>
       <c r="I51" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J51">
         <v>1</v>
@@ -2773,10 +2749,10 @@
         <v>1.8</v>
       </c>
       <c r="M51">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13">
       <c r="A52" s="1">
         <v>209</v>
       </c>
@@ -2793,7 +2769,7 @@
         <v>-0.3</v>
       </c>
       <c r="F52">
-        <v>-0.17499999999999999</v>
+        <v>-0.175</v>
       </c>
       <c r="G52">
         <v>6</v>
@@ -2802,7 +2778,7 @@
         <v>1</v>
       </c>
       <c r="I52" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J52">
         <v>1</v>
@@ -2811,10 +2787,10 @@
         <v>1.8</v>
       </c>
       <c r="M52">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13">
       <c r="A53" s="1">
         <v>216</v>
       </c>
@@ -2840,7 +2816,7 @@
         <v>1</v>
       </c>
       <c r="I53" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J53">
         <v>1</v>
@@ -2852,7 +2828,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:13">
       <c r="A54" s="1">
         <v>230</v>
       </c>
@@ -2869,7 +2845,7 @@
         <v>0.6</v>
       </c>
       <c r="F54">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.025</v>
       </c>
       <c r="G54" t="s">
         <v>86</v>
@@ -2878,7 +2854,7 @@
         <v>1</v>
       </c>
       <c r="I54" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J54">
         <v>1</v>
@@ -2890,7 +2866,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13">
       <c r="A55" s="1">
         <v>212</v>
       </c>
@@ -2916,7 +2892,7 @@
         <v>1</v>
       </c>
       <c r="I55" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J55">
         <v>1</v>
@@ -2928,7 +2904,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:13">
       <c r="A56" s="1">
         <v>213</v>
       </c>
@@ -2954,7 +2930,7 @@
         <v>1</v>
       </c>
       <c r="I56" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J56">
         <v>1</v>
@@ -2966,7 +2942,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:13">
       <c r="A57" s="1">
         <v>214</v>
       </c>
@@ -2992,7 +2968,7 @@
         <v>1</v>
       </c>
       <c r="I57" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J57">
         <v>1</v>
@@ -3004,7 +2980,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:13">
       <c r="A58" s="1">
         <v>215</v>
       </c>
@@ -3030,7 +3006,7 @@
         <v>1</v>
       </c>
       <c r="I58" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J58">
         <v>1</v>
@@ -3042,7 +3018,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13">
       <c r="A59" s="1">
         <v>217</v>
       </c>
@@ -3068,7 +3044,7 @@
         <v>1</v>
       </c>
       <c r="I59" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J59">
         <v>1</v>
@@ -3080,7 +3056,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:13">
       <c r="A60" s="1">
         <v>218</v>
       </c>
@@ -3106,7 +3082,7 @@
         <v>1</v>
       </c>
       <c r="I60" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J60">
         <v>1</v>
@@ -3118,7 +3094,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:13">
       <c r="A61" s="1">
         <v>231</v>
       </c>
@@ -3135,7 +3111,7 @@
         <v>1.2</v>
       </c>
       <c r="F61">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.025</v>
       </c>
       <c r="G61" t="s">
         <v>86</v>
@@ -3144,7 +3120,7 @@
         <v>1</v>
       </c>
       <c r="I61" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J61">
         <v>1</v>
@@ -3156,7 +3132,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:13">
       <c r="A62" s="1">
         <v>219</v>
       </c>
@@ -3182,7 +3158,7 @@
         <v>1</v>
       </c>
       <c r="I62" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J62">
         <v>1</v>
@@ -3194,7 +3170,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:13">
       <c r="A63" s="1">
         <v>221</v>
       </c>
@@ -3220,7 +3196,7 @@
         <v>1</v>
       </c>
       <c r="I63" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J63">
         <v>1</v>
@@ -3232,7 +3208,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:13">
       <c r="A64" s="1">
         <v>222</v>
       </c>
@@ -3258,7 +3234,7 @@
         <v>1</v>
       </c>
       <c r="I64" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J64">
         <v>1</v>
@@ -3270,7 +3246,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13">
       <c r="A65" s="1">
         <v>223</v>
       </c>
@@ -3296,7 +3272,7 @@
         <v>1</v>
       </c>
       <c r="I65" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J65">
         <v>1</v>
@@ -3308,7 +3284,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13">
       <c r="A66" s="1">
         <v>224</v>
       </c>
@@ -3334,7 +3310,7 @@
         <v>1</v>
       </c>
       <c r="I66" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J66">
         <v>1</v>
@@ -3346,7 +3322,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13">
       <c r="A67" s="1">
         <v>225</v>
       </c>
@@ -3372,7 +3348,7 @@
         <v>1</v>
       </c>
       <c r="I67" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J67">
         <v>1</v>
@@ -3384,7 +3360,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13">
       <c r="A68" s="1">
         <v>226</v>
       </c>
@@ -3401,7 +3377,7 @@
         <v>0.6</v>
       </c>
       <c r="F68">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.025</v>
       </c>
       <c r="G68" t="s">
         <v>86</v>
@@ -3410,7 +3386,7 @@
         <v>1</v>
       </c>
       <c r="I68" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J68">
         <v>1</v>
@@ -3422,7 +3398,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13">
       <c r="A69" s="1">
         <v>227</v>
       </c>
@@ -3439,7 +3415,7 @@
         <v>1.2</v>
       </c>
       <c r="F69">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.025</v>
       </c>
       <c r="G69" t="s">
         <v>86</v>
@@ -3448,7 +3424,7 @@
         <v>1</v>
       </c>
       <c r="I69" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J69">
         <v>1</v>
@@ -3460,7 +3436,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13">
       <c r="A70" s="1">
         <v>228</v>
       </c>
@@ -3471,13 +3447,13 @@
         <v>83</v>
       </c>
       <c r="D70">
-        <v>2.0099999999999998</v>
+        <v>2.01</v>
       </c>
       <c r="E70">
         <v>0.6</v>
       </c>
       <c r="F70">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.025</v>
       </c>
       <c r="G70" t="s">
         <v>86</v>
@@ -3486,7 +3462,7 @@
         <v>1</v>
       </c>
       <c r="I70" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J70">
         <v>1</v>
@@ -3498,7 +3474,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13">
       <c r="A71" s="1">
         <v>229</v>
       </c>
@@ -3509,13 +3485,13 @@
         <v>84</v>
       </c>
       <c r="D71">
-        <v>2.0099999999999998</v>
+        <v>2.01</v>
       </c>
       <c r="E71">
         <v>1.2</v>
       </c>
       <c r="F71">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.025</v>
       </c>
       <c r="G71" t="s">
         <v>86</v>
@@ -3524,7 +3500,7 @@
         <v>1</v>
       </c>
       <c r="I71" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J71">
         <v>1</v>
@@ -3536,7 +3512,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13">
       <c r="A72" s="1">
         <v>220</v>
       </c>
@@ -3562,7 +3538,7 @@
         <v>1</v>
       </c>
       <c r="I72" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J72">
         <v>1</v>
@@ -3580,25 +3556,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="78.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.28515625" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3642,15 +3604,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15">
       <c r="A2" s="1">
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -3659,7 +3621,7 @@
         <v>0.06</v>
       </c>
       <c r="F2">
-        <v>0.17499999999999999</v>
+        <v>0.175</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -3668,7 +3630,7 @@
         <v>6</v>
       </c>
       <c r="I2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -3677,18 +3639,18 @@
         <v>2.76</v>
       </c>
       <c r="M2">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
       <c r="A3" s="1">
         <v>235</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -3697,7 +3659,7 @@
         <v>-0.255</v>
       </c>
       <c r="F3">
-        <v>0.13700000000000001</v>
+        <v>0.137</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -3706,7 +3668,7 @@
         <v>6</v>
       </c>
       <c r="I3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -3715,18 +3677,18 @@
         <v>2.76</v>
       </c>
       <c r="M3">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
       <c r="A4" s="1">
         <v>234</v>
       </c>
       <c r="B4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -3735,7 +3697,7 @@
         <v>0.375</v>
       </c>
       <c r="F4">
-        <v>0.13700000000000001</v>
+        <v>0.137</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -3744,7 +3706,7 @@
         <v>6</v>
       </c>
       <c r="I4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -3753,18 +3715,18 @@
         <v>2.76</v>
       </c>
       <c r="M4">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
       <c r="A5" s="1">
         <v>233</v>
       </c>
       <c r="B5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -3773,7 +3735,7 @@
         <v>-0.255</v>
       </c>
       <c r="F5">
-        <v>0.21299999999999999</v>
+        <v>0.213</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -3782,7 +3744,7 @@
         <v>6</v>
       </c>
       <c r="I5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -3791,18 +3753,18 @@
         <v>2.76</v>
       </c>
       <c r="M5">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6" s="1">
         <v>232</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -3811,7 +3773,7 @@
         <v>0.375</v>
       </c>
       <c r="F6">
-        <v>0.21299999999999999</v>
+        <v>0.213</v>
       </c>
       <c r="G6">
         <v>1</v>
@@ -3820,7 +3782,7 @@
         <v>6</v>
       </c>
       <c r="I6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -3829,27 +3791,27 @@
         <v>2.76</v>
       </c>
       <c r="M6">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
       <c r="A7" s="1">
         <v>242</v>
       </c>
       <c r="B7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D7">
         <v>0.6</v>
       </c>
       <c r="E7">
-        <v>-0.79500000000000004</v>
+        <v>-0.795</v>
       </c>
       <c r="F7">
-        <v>-8.5999999999999993E-2</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="G7">
         <v>3</v>
@@ -3858,7 +3820,7 @@
         <v>6</v>
       </c>
       <c r="I7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -3867,18 +3829,18 @@
         <v>0.96</v>
       </c>
       <c r="M7">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8" s="1">
         <v>236</v>
       </c>
       <c r="B8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D8">
         <v>0.6</v>
@@ -3887,7 +3849,7 @@
         <v>-1.012</v>
       </c>
       <c r="F8">
-        <v>0.96199999999999997</v>
+        <v>0.962</v>
       </c>
       <c r="G8">
         <v>3</v>
@@ -3896,7 +3858,7 @@
         <v>6</v>
       </c>
       <c r="I8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -3905,27 +3867,27 @@
         <v>0.96</v>
       </c>
       <c r="M8">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
       <c r="A9" s="1">
         <v>237</v>
       </c>
       <c r="B9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D9">
         <v>0.6</v>
       </c>
       <c r="E9">
-        <v>-0.81200000000000006</v>
+        <v>-0.8120000000000001</v>
       </c>
       <c r="F9">
-        <v>0.96199999999999997</v>
+        <v>0.962</v>
       </c>
       <c r="G9">
         <v>3</v>
@@ -3934,7 +3896,7 @@
         <v>6</v>
       </c>
       <c r="I9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J9">
         <v>1</v>
@@ -3943,18 +3905,18 @@
         <v>0.96</v>
       </c>
       <c r="M9">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10" s="1">
         <v>238</v>
       </c>
       <c r="B10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D10">
         <v>0.6</v>
@@ -3972,7 +3934,7 @@
         <v>6</v>
       </c>
       <c r="I10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J10">
         <v>1</v>
@@ -3981,24 +3943,24 @@
         <v>0.96</v>
       </c>
       <c r="M10">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
       <c r="A11" s="1">
         <v>239</v>
       </c>
       <c r="B11" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C11" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D11">
         <v>0.6</v>
       </c>
       <c r="E11">
-        <v>-0.81200000000000006</v>
+        <v>-0.8120000000000001</v>
       </c>
       <c r="F11">
         <v>-0.188</v>
@@ -4010,7 +3972,7 @@
         <v>6</v>
       </c>
       <c r="I11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J11">
         <v>1</v>
@@ -4019,27 +3981,27 @@
         <v>0.96</v>
       </c>
       <c r="M11">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
       <c r="A12" s="1">
         <v>240</v>
       </c>
       <c r="B12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D12">
         <v>0.6</v>
       </c>
       <c r="E12">
-        <v>-0.79500000000000004</v>
+        <v>-0.795</v>
       </c>
       <c r="F12">
-        <v>-1.4E-2</v>
+        <v>-0.014</v>
       </c>
       <c r="G12">
         <v>3</v>
@@ -4048,7 +4010,7 @@
         <v>6</v>
       </c>
       <c r="I12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J12">
         <v>1</v>
@@ -4057,27 +4019,27 @@
         <v>0.96</v>
       </c>
       <c r="M12">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
       <c r="A13" s="1">
         <v>241</v>
       </c>
       <c r="B13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D13">
         <v>0.6</v>
       </c>
       <c r="E13">
-        <v>-0.65500000000000003</v>
+        <v>-0.655</v>
       </c>
       <c r="F13">
-        <v>-1.4E-2</v>
+        <v>-0.014</v>
       </c>
       <c r="G13">
         <v>3</v>
@@ -4086,7 +4048,7 @@
         <v>6</v>
       </c>
       <c r="I13" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J13">
         <v>1</v>
@@ -4095,27 +4057,27 @@
         <v>0.96</v>
       </c>
       <c r="M13">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
       <c r="A14" s="1">
         <v>160</v>
       </c>
       <c r="B14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D14">
         <v>0.6</v>
       </c>
       <c r="E14">
-        <v>-0.91200000000000003</v>
+        <v>-0.912</v>
       </c>
       <c r="F14">
-        <v>0.38700000000000001</v>
+        <v>0.387</v>
       </c>
       <c r="G14">
         <v>3</v>
@@ -4124,7 +4086,7 @@
         <v>6</v>
       </c>
       <c r="I14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J14">
         <v>1</v>
@@ -4133,27 +4095,27 @@
         <v>0.96</v>
       </c>
       <c r="M14">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
       <c r="A15" s="1">
         <v>243</v>
       </c>
       <c r="B15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C15" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D15">
         <v>0.6</v>
       </c>
       <c r="E15">
-        <v>-0.65500000000000003</v>
+        <v>-0.655</v>
       </c>
       <c r="F15">
-        <v>-8.5999999999999993E-2</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="G15">
         <v>3</v>
@@ -4162,7 +4124,7 @@
         <v>6</v>
       </c>
       <c r="I15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J15">
         <v>1</v>
@@ -4171,24 +4133,24 @@
         <v>0.96</v>
       </c>
       <c r="M15">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
       <c r="A16" s="1">
         <v>92</v>
       </c>
       <c r="B16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D16">
         <v>0.6</v>
       </c>
       <c r="E16">
-        <v>-0.72499999999999998</v>
+        <v>-0.725</v>
       </c>
       <c r="F16">
         <v>-0.05</v>
@@ -4200,7 +4162,7 @@
         <v>6</v>
       </c>
       <c r="I16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J16">
         <v>1</v>
@@ -4209,24 +4171,24 @@
         <v>0.96</v>
       </c>
       <c r="M16">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17" s="1">
         <v>245</v>
       </c>
       <c r="B17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C17" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D17">
         <v>0.96</v>
       </c>
       <c r="E17">
-        <v>0.45500000000000002</v>
+        <v>0.455</v>
       </c>
       <c r="F17">
         <v>-0.375</v>
@@ -4238,7 +4200,7 @@
         <v>6</v>
       </c>
       <c r="I17" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J17">
         <v>1</v>
@@ -4247,18 +4209,18 @@
         <v>0.6</v>
       </c>
       <c r="M17">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
       <c r="A18" s="1">
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D18">
         <v>0.96</v>
@@ -4276,7 +4238,7 @@
         <v>6</v>
       </c>
       <c r="I18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J18">
         <v>1</v>
@@ -4285,24 +4247,24 @@
         <v>0.6</v>
       </c>
       <c r="M18">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
       <c r="A19" s="1">
         <v>244</v>
       </c>
       <c r="B19" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C19" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D19">
         <v>0.96</v>
       </c>
       <c r="E19">
-        <v>0.40500000000000003</v>
+        <v>0.405</v>
       </c>
       <c r="F19">
         <v>-0.375</v>
@@ -4314,7 +4276,7 @@
         <v>6</v>
       </c>
       <c r="I19" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J19">
         <v>1</v>
@@ -4323,18 +4285,18 @@
         <v>0.6</v>
       </c>
       <c r="M19">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
       <c r="A20" s="1">
         <v>256</v>
       </c>
       <c r="B20" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -4352,7 +4314,7 @@
         <v>6</v>
       </c>
       <c r="I20" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J20">
         <v>1</v>
@@ -4361,18 +4323,18 @@
         <v>1.8</v>
       </c>
       <c r="M20">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
       <c r="A21" s="1">
         <v>258</v>
       </c>
       <c r="B21" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C21" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D21">
         <v>0</v>
@@ -4390,7 +4352,7 @@
         <v>6</v>
       </c>
       <c r="I21" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J21">
         <v>1</v>
@@ -4399,18 +4361,18 @@
         <v>1.8</v>
       </c>
       <c r="M21">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
       <c r="A22" s="1">
         <v>259</v>
       </c>
       <c r="B22" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C22" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -4428,7 +4390,7 @@
         <v>6</v>
       </c>
       <c r="I22" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J22">
         <v>1</v>
@@ -4437,18 +4399,18 @@
         <v>1.8</v>
       </c>
       <c r="M22">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13">
       <c r="A23" s="1">
         <v>260</v>
       </c>
       <c r="B23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C23" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -4466,7 +4428,7 @@
         <v>6</v>
       </c>
       <c r="I23" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J23">
         <v>1</v>
@@ -4475,18 +4437,18 @@
         <v>1.8</v>
       </c>
       <c r="M23">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
       <c r="A24" s="1">
         <v>261</v>
       </c>
       <c r="B24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C24" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D24">
         <v>0</v>
@@ -4504,7 +4466,7 @@
         <v>6</v>
       </c>
       <c r="I24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J24">
         <v>1</v>
@@ -4513,18 +4475,18 @@
         <v>1.8</v>
       </c>
       <c r="M24">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13">
       <c r="A25" s="1">
         <v>257</v>
       </c>
       <c r="B25" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C25" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -4542,7 +4504,7 @@
         <v>6</v>
       </c>
       <c r="I25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J25">
         <v>1</v>
@@ -4551,24 +4513,24 @@
         <v>1.8</v>
       </c>
       <c r="M25">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13">
       <c r="A26" s="1">
         <v>250</v>
       </c>
       <c r="B26" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C26" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D26">
-        <v>8.7999999999999995E-2</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="E26">
-        <v>2.5000000000000001E-2</v>
+        <v>0.025</v>
       </c>
       <c r="F26">
         <v>-0.22</v>
@@ -4580,7 +4542,7 @@
         <v>6</v>
       </c>
       <c r="I26" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J26">
         <v>1</v>
@@ -4589,18 +4551,18 @@
         <v>1.8</v>
       </c>
       <c r="M26">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
       <c r="A27" s="1">
         <v>252</v>
       </c>
       <c r="B27" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C27" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D27">
         <v>0.183</v>
@@ -4609,7 +4571,7 @@
         <v>0.21</v>
       </c>
       <c r="F27">
-        <v>-0.40200000000000002</v>
+        <v>-0.402</v>
       </c>
       <c r="G27">
         <v>5</v>
@@ -4618,7 +4580,7 @@
         <v>6</v>
       </c>
       <c r="I27" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J27">
         <v>1</v>
@@ -4627,27 +4589,27 @@
         <v>1.8</v>
       </c>
       <c r="M27">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13">
       <c r="A28" s="1">
         <v>246</v>
       </c>
       <c r="B28" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C28" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D28">
-        <v>8.7999999999999995E-2</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="E28">
-        <v>-0.22500000000000001</v>
+        <v>-0.225</v>
       </c>
       <c r="F28">
-        <v>2.5999999999999999E-2</v>
+        <v>0.026</v>
       </c>
       <c r="G28">
         <v>5</v>
@@ -4656,7 +4618,7 @@
         <v>6</v>
       </c>
       <c r="I28" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J28">
         <v>1</v>
@@ -4665,27 +4627,27 @@
         <v>1.8</v>
       </c>
       <c r="M28">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
       <c r="A29" s="1">
         <v>247</v>
       </c>
       <c r="B29" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C29" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D29">
-        <v>8.7999999999999995E-2</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="E29">
-        <v>0.27500000000000002</v>
+        <v>0.275</v>
       </c>
       <c r="F29">
-        <v>2.5999999999999999E-2</v>
+        <v>0.026</v>
       </c>
       <c r="G29">
         <v>5</v>
@@ -4694,7 +4656,7 @@
         <v>6</v>
       </c>
       <c r="I29" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J29">
         <v>1</v>
@@ -4703,27 +4665,27 @@
         <v>1.8</v>
       </c>
       <c r="M29">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
       <c r="A30" s="1">
         <v>248</v>
       </c>
       <c r="B30" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C30" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D30">
-        <v>8.7999999999999995E-2</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="E30">
-        <v>-0.22500000000000001</v>
+        <v>-0.225</v>
       </c>
       <c r="F30">
-        <v>-0.46600000000000003</v>
+        <v>-0.466</v>
       </c>
       <c r="G30">
         <v>5</v>
@@ -4732,7 +4694,7 @@
         <v>6</v>
       </c>
       <c r="I30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J30">
         <v>1</v>
@@ -4741,27 +4703,27 @@
         <v>1.8</v>
       </c>
       <c r="M30">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
       <c r="A31" s="1">
         <v>249</v>
       </c>
       <c r="B31" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C31" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D31">
-        <v>8.7999999999999995E-2</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="E31">
-        <v>0.27500000000000002</v>
+        <v>0.275</v>
       </c>
       <c r="F31">
-        <v>-0.46600000000000003</v>
+        <v>-0.466</v>
       </c>
       <c r="G31">
         <v>5</v>
@@ -4770,7 +4732,7 @@
         <v>6</v>
       </c>
       <c r="I31" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J31">
         <v>1</v>
@@ -4779,18 +4741,18 @@
         <v>1.8</v>
       </c>
       <c r="M31">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13">
       <c r="A32" s="1">
         <v>251</v>
       </c>
       <c r="B32" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C32" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D32">
         <v>0.183</v>
@@ -4799,7 +4761,7 @@
         <v>-0.15</v>
       </c>
       <c r="F32">
-        <v>-0.40200000000000002</v>
+        <v>-0.402</v>
       </c>
       <c r="G32">
         <v>5</v>
@@ -4808,7 +4770,7 @@
         <v>6</v>
       </c>
       <c r="I32" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J32">
         <v>1</v>
@@ -4817,18 +4779,18 @@
         <v>1.8</v>
       </c>
       <c r="M32">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13">
       <c r="A33" s="1">
         <v>262</v>
       </c>
       <c r="B33" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C33" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D33">
         <v>0</v>
@@ -4846,7 +4808,7 @@
         <v>6</v>
       </c>
       <c r="I33" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J33">
         <v>1</v>
@@ -4855,18 +4817,18 @@
         <v>1.8</v>
       </c>
       <c r="M33">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13">
       <c r="A34" s="1">
         <v>253</v>
       </c>
       <c r="B34" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C34" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D34">
         <v>0.183</v>
@@ -4884,7 +4846,7 @@
         <v>6</v>
       </c>
       <c r="I34" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J34">
         <v>1</v>
@@ -4893,18 +4855,18 @@
         <v>1.8</v>
       </c>
       <c r="M34">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13">
       <c r="A35" s="1">
         <v>263</v>
       </c>
       <c r="B35" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C35" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D35">
         <v>0</v>
@@ -4922,7 +4884,7 @@
         <v>6</v>
       </c>
       <c r="I35" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J35">
         <v>1</v>
@@ -4931,18 +4893,18 @@
         <v>1.8</v>
       </c>
       <c r="M35">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13">
       <c r="A36" s="1">
         <v>255</v>
       </c>
       <c r="B36" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C36" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D36">
         <v>0.183</v>
@@ -4951,7 +4913,7 @@
         <v>0.03</v>
       </c>
       <c r="F36">
-        <v>-0.61599999999999999</v>
+        <v>-0.616</v>
       </c>
       <c r="G36">
         <v>5</v>
@@ -4960,7 +4922,7 @@
         <v>6</v>
       </c>
       <c r="I36" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J36">
         <v>1</v>
@@ -4969,18 +4931,18 @@
         <v>1.8</v>
       </c>
       <c r="M36">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
       <c r="A37" s="1">
         <v>156</v>
       </c>
       <c r="B37" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C37" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D37">
         <v>0.108</v>
@@ -4989,7 +4951,7 @@
         <v>0.03</v>
       </c>
       <c r="F37">
-        <v>-0.17499999999999999</v>
+        <v>-0.175</v>
       </c>
       <c r="G37">
         <v>5</v>
@@ -4998,7 +4960,7 @@
         <v>6</v>
       </c>
       <c r="I37" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J37">
         <v>1</v>
@@ -5007,24 +4969,24 @@
         <v>1.8</v>
       </c>
       <c r="M37">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13">
       <c r="A38" s="1">
         <v>158</v>
       </c>
       <c r="B38" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C38" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D38">
-        <v>0.20799999999999999</v>
+        <v>0.208</v>
       </c>
       <c r="E38">
-        <v>-9.5000000000000001E-2</v>
+        <v>-0.095</v>
       </c>
       <c r="F38">
         <v>-1.024</v>
@@ -5036,7 +4998,7 @@
         <v>6</v>
       </c>
       <c r="I38" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J38">
         <v>1</v>
@@ -5045,18 +5007,18 @@
         <v>1.8</v>
       </c>
       <c r="M38">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13">
       <c r="A39" s="1">
         <v>254</v>
       </c>
       <c r="B39" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C39" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D39">
         <v>0.183</v>
@@ -5074,7 +5036,7 @@
         <v>6</v>
       </c>
       <c r="I39" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J39">
         <v>1</v>
@@ -5083,24 +5045,24 @@
         <v>1.8</v>
       </c>
       <c r="M39">
-        <v>2.6549999999999998</v>
-      </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+        <v>2.655</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13">
       <c r="A40" s="1">
         <v>264</v>
       </c>
       <c r="B40" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C40" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D40">
-        <v>0.56999999999999995</v>
+        <v>0.57</v>
       </c>
       <c r="E40">
-        <v>1.1499999999999999</v>
+        <v>1.15</v>
       </c>
       <c r="F40">
         <v>-0.05</v>
@@ -5112,7 +5074,7 @@
         <v>6</v>
       </c>
       <c r="I40" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J40">
         <v>1</v>
@@ -5124,18 +5086,18 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13">
       <c r="A41" s="1">
         <v>266</v>
       </c>
       <c r="B41" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C41" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D41">
-        <v>0.56999999999999995</v>
+        <v>0.57</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -5150,7 +5112,7 @@
         <v>6</v>
       </c>
       <c r="I41" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J41">
         <v>1</v>
@@ -5162,15 +5124,15 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13">
       <c r="A42" s="1">
         <v>277</v>
       </c>
       <c r="B42" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C42" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D42">
         <v>1.06</v>
@@ -5179,7 +5141,7 @@
         <v>1.585</v>
       </c>
       <c r="F42">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.025</v>
       </c>
       <c r="G42" t="s">
         <v>86</v>
@@ -5188,7 +5150,7 @@
         <v>6</v>
       </c>
       <c r="I42" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J42">
         <v>1</v>
@@ -5200,15 +5162,15 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13">
       <c r="A43" s="1">
         <v>267</v>
       </c>
       <c r="B43" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C43" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D43">
         <v>0.72</v>
@@ -5226,7 +5188,7 @@
         <v>6</v>
       </c>
       <c r="I43" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J43">
         <v>1</v>
@@ -5238,15 +5200,15 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13">
       <c r="A44" s="1">
         <v>276</v>
       </c>
       <c r="B44" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C44" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D44">
         <v>0.96</v>
@@ -5255,7 +5217,7 @@
         <v>1.585</v>
       </c>
       <c r="F44">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.025</v>
       </c>
       <c r="G44" t="s">
         <v>86</v>
@@ -5264,7 +5226,7 @@
         <v>6</v>
       </c>
       <c r="I44" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J44">
         <v>1</v>
@@ -5276,24 +5238,24 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13">
       <c r="A45" s="1">
         <v>270</v>
       </c>
       <c r="B45" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C45" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D45">
         <v>0.96</v>
       </c>
       <c r="E45">
-        <v>1.4850000000000001</v>
+        <v>1.485</v>
       </c>
       <c r="F45">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.025</v>
       </c>
       <c r="G45" t="s">
         <v>86</v>
@@ -5302,7 +5264,7 @@
         <v>6</v>
       </c>
       <c r="I45" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J45">
         <v>1</v>
@@ -5314,24 +5276,24 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13">
       <c r="A46" s="1">
         <v>271</v>
       </c>
       <c r="B46" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C46" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D46">
         <v>1.06</v>
       </c>
       <c r="E46">
-        <v>1.4850000000000001</v>
+        <v>1.485</v>
       </c>
       <c r="F46">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.025</v>
       </c>
       <c r="G46" t="s">
         <v>86</v>
@@ -5340,7 +5302,7 @@
         <v>6</v>
       </c>
       <c r="I46" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J46">
         <v>1</v>
@@ -5352,21 +5314,21 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13">
       <c r="A47" s="1">
         <v>273</v>
       </c>
       <c r="B47" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C47" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D47">
         <v>0.72</v>
       </c>
       <c r="E47">
-        <v>1.1499999999999999</v>
+        <v>1.15</v>
       </c>
       <c r="F47">
         <v>-0.05</v>
@@ -5378,7 +5340,7 @@
         <v>6</v>
       </c>
       <c r="I47" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J47">
         <v>1</v>
@@ -5390,24 +5352,24 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13">
       <c r="A48" s="1">
         <v>157</v>
       </c>
       <c r="B48" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C48" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D48">
         <v>1.01</v>
       </c>
       <c r="E48">
-        <v>1.5349999999999999</v>
+        <v>1.535</v>
       </c>
       <c r="F48">
-        <v>-2.5000000000000001E-2</v>
+        <v>-0.025</v>
       </c>
       <c r="G48" t="s">
         <v>86</v>
@@ -5416,7 +5378,7 @@
         <v>6</v>
       </c>
       <c r="I48" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J48">
         <v>1</v>
@@ -5428,18 +5390,18 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13">
       <c r="A49" s="1">
         <v>159</v>
       </c>
       <c r="B49" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C49" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D49">
-        <v>0.64500000000000002</v>
+        <v>0.645</v>
       </c>
       <c r="E49">
         <v>1.075</v>
@@ -5454,7 +5416,7 @@
         <v>6</v>
       </c>
       <c r="I49" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J49">
         <v>1</v>
@@ -5472,31 +5434,31 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="B1:O1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:15">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>7</v>

</xml_diff>